<commit_message>
add -0.7 muzzle loudness for subsonic ammo
</commit_message>
<xml_diff>
--- a/changes/308-ammo-super.xlsx
+++ b/changes/308-ammo-super.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A1B1931-2D90-4139-9ED7-B2833B0B5A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9634F945-6EDF-425D-959F-1E17C4F27852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="7.62x51-ammo" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
     <author/>
   </authors>
   <commentList>
-    <comment ref="L2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
+    <comment ref="M2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000003000000}">
       <text>
         <r>
           <rPr>
@@ -55,7 +55,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
+    <comment ref="T2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
       <text>
         <r>
           <rPr>
@@ -71,7 +71,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AI2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+    <comment ref="AJ2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
       <text>
         <r>
           <rPr>
@@ -118,7 +118,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="104">
   <si>
     <t>7.62x51 ammo scoring model</t>
   </si>
@@ -424,6 +424,12 @@
   </si>
   <si>
     <t>7.62x51_appalachian_m62_142gr_red_tracer</t>
+  </si>
+  <si>
+    <t>muzzle_loudness</t>
+  </si>
+  <si>
+    <t>yeah</t>
   </si>
 </sst>
 </file>
@@ -725,7 +731,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -874,11 +880,17 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -888,21 +900,44 @@
     <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FF1F2933"/>
+        <name val="Carlito"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -930,9 +965,9 @@
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="7.62x51-ammo-style" pivot="0" count="3" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="headerRow" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="secondRowStripe" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -947,8 +982,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="A2:AQ21">
-  <tableColumns count="43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="A2:AR21">
+  <tableColumns count="44">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="name"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="pretty_name"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="ergonomics"/>
@@ -959,6 +994,7 @@
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="bullet_damage"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="bullet_velocity"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="fire_rate"/>
+    <tableColumn id="44" xr3:uid="{7C52D374-9102-4BD4-8011-A11751C9A1CF}" name="muzzle_loudness" dataDxfId="0"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="price"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="damage_torso_a"/>
     <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="damage_torso_b"/>
@@ -1195,80 +1231,81 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AQ998"/>
+  <dimension ref="A1:AR998"/>
   <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="19.625" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
     <col min="3" max="8" width="5.625" customWidth="1"/>
     <col min="9" max="9" width="8" customWidth="1"/>
-    <col min="10" max="28" width="5.625" customWidth="1"/>
-    <col min="29" max="29" width="24.875" customWidth="1"/>
-    <col min="30" max="36" width="5.625" customWidth="1"/>
-    <col min="37" max="37" width="9.625" customWidth="1"/>
-    <col min="38" max="43" width="5.625" customWidth="1"/>
+    <col min="10" max="29" width="5.625" customWidth="1"/>
+    <col min="30" max="30" width="24.875" customWidth="1"/>
+    <col min="31" max="37" width="5.625" customWidth="1"/>
+    <col min="38" max="38" width="9.625" customWidth="1"/>
+    <col min="39" max="44" width="5.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="24" customHeight="1">
-      <c r="A1" s="58" t="s">
+    <row r="1" spans="1:44" ht="24" customHeight="1">
+      <c r="A1" s="62" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="59"/>
-      <c r="E1" s="59"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="61" t="s">
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="59"/>
+      <c r="M1" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="M1" s="59"/>
-      <c r="N1" s="59"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="13"/>
+      <c r="N1" s="61"/>
+      <c r="O1" s="61"/>
+      <c r="P1" s="59"/>
       <c r="Q1" s="13"/>
       <c r="R1" s="13"/>
-      <c r="S1" s="62" t="s">
+      <c r="S1" s="13"/>
+      <c r="T1" s="64" t="s">
         <v>26</v>
       </c>
-      <c r="T1" s="59"/>
-      <c r="U1" s="59"/>
-      <c r="V1" s="59"/>
-      <c r="W1" s="59"/>
-      <c r="X1" s="59"/>
-      <c r="Y1" s="59"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="61" t="s">
+      <c r="U1" s="61"/>
+      <c r="V1" s="61"/>
+      <c r="W1" s="61"/>
+      <c r="X1" s="61"/>
+      <c r="Y1" s="61"/>
+      <c r="Z1" s="61"/>
+      <c r="AA1" s="59"/>
+      <c r="AB1" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="AB1" s="59"/>
-      <c r="AC1" s="59"/>
-      <c r="AD1" s="59"/>
-      <c r="AE1" s="59"/>
-      <c r="AF1" s="59"/>
-      <c r="AG1" s="60"/>
-      <c r="AH1" s="63" t="s">
+      <c r="AC1" s="61"/>
+      <c r="AD1" s="61"/>
+      <c r="AE1" s="61"/>
+      <c r="AF1" s="61"/>
+      <c r="AG1" s="61"/>
+      <c r="AH1" s="59"/>
+      <c r="AI1" s="65" t="s">
         <v>28</v>
       </c>
-      <c r="AI1" s="60"/>
-      <c r="AJ1" s="64" t="s">
+      <c r="AJ1" s="59"/>
+      <c r="AK1" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="AK1" s="60"/>
-      <c r="AL1" s="65" t="s">
+      <c r="AL1" s="59"/>
+      <c r="AM1" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="AM1" s="59"/>
-      <c r="AN1" s="59"/>
-      <c r="AO1" s="59"/>
-      <c r="AP1" s="59"/>
-      <c r="AQ1" s="60"/>
-    </row>
-    <row r="2" spans="1:43" ht="45.75" customHeight="1">
+      <c r="AN1" s="61"/>
+      <c r="AO1" s="61"/>
+      <c r="AP1" s="61"/>
+      <c r="AQ1" s="61"/>
+      <c r="AR1" s="59"/>
+    </row>
+    <row r="2" spans="1:44" ht="45.75" customHeight="1">
       <c r="A2" s="16" t="s">
         <v>36</v>
       </c>
@@ -1300,106 +1337,109 @@
         <v>44</v>
       </c>
       <c r="K2" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="L2" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="L2" s="16" t="s">
+      <c r="M2" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="M2" s="16" t="s">
+      <c r="N2" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="N2" s="16" t="s">
+      <c r="O2" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="O2" s="16" t="s">
+      <c r="P2" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="P2" s="16" t="s">
+      <c r="Q2" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="Q2" s="16" t="s">
+      <c r="R2" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="R2" s="16" t="s">
+      <c r="S2" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="S2" s="16" t="s">
+      <c r="T2" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="T2" s="16" t="s">
+      <c r="U2" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="U2" s="16" t="s">
+      <c r="V2" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="V2" s="16" t="s">
+      <c r="W2" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="W2" s="16" t="s">
+      <c r="X2" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="X2" s="16" t="s">
+      <c r="Y2" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="Y2" s="16" t="s">
+      <c r="Z2" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="Z2" s="16" t="s">
+      <c r="AA2" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="AA2" s="16" t="s">
+      <c r="AB2" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="AB2" s="16" t="s">
+      <c r="AC2" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="AC2" s="16" t="s">
+      <c r="AD2" s="16" t="s">
         <v>65</v>
       </c>
-      <c r="AD2" s="16" t="s">
+      <c r="AE2" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="AE2" s="16" t="s">
+      <c r="AF2" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="AF2" s="16" t="s">
+      <c r="AG2" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="AG2" s="16" t="s">
+      <c r="AH2" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="AH2" s="16" t="s">
+      <c r="AI2" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="AI2" s="16" t="s">
+      <c r="AJ2" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="AJ2" s="16" t="s">
+      <c r="AK2" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="AK2" s="16" t="s">
+      <c r="AL2" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="AL2" s="16" t="s">
+      <c r="AM2" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="AM2" s="16" t="s">
+      <c r="AN2" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="AN2" s="16" t="s">
+      <c r="AO2" s="16" t="s">
         <v>79</v>
       </c>
-      <c r="AO2" s="16" t="s">
+      <c r="AP2" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="AP2" s="16" t="s">
+      <c r="AQ2" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="AQ2" s="16" t="s">
+      <c r="AR2" s="16" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:43" ht="14.25" customHeight="1">
+    <row r="3" spans="1:44" ht="14.25" customHeight="1">
       <c r="A3" s="23" t="s">
         <v>100</v>
       </c>
@@ -1426,124 +1466,125 @@
         <v>0</v>
       </c>
       <c r="J3" s="28"/>
-      <c r="K3" s="29">
+      <c r="K3" s="28"/>
+      <c r="L3" s="29">
         <v>0</v>
       </c>
-      <c r="L3" s="30">
+      <c r="M3" s="30">
         <v>-2.5999999999999999E-2</v>
       </c>
-      <c r="M3" s="30">
+      <c r="N3" s="30">
         <v>104.5</v>
       </c>
-      <c r="N3" s="30">
+      <c r="O3" s="30">
         <v>104</v>
       </c>
-      <c r="O3" s="30">
+      <c r="P3" s="30">
         <v>1</v>
       </c>
-      <c r="P3" s="30">
+      <c r="Q3" s="30">
         <v>0.3</v>
       </c>
-      <c r="Q3" s="30">
+      <c r="R3" s="30">
         <v>0.5</v>
       </c>
-      <c r="R3" s="31">
+      <c r="S3" s="31">
         <v>2.5</v>
       </c>
-      <c r="S3" s="32">
-        <f>MAX(MIN($L3*Model!$A$13+$M3,$N3)*$O3,0)</f>
+      <c r="T3" s="32">
+        <f>MAX(MIN($M3*Model!$A$13+$N3,$O3)*$P3,0)</f>
         <v>103.85</v>
       </c>
-      <c r="T3" s="32">
-        <f>MAX(MIN($L3*Model!$A$14+$M3,$N3)*$O3,0)</f>
+      <c r="U3" s="32">
+        <f>MAX(MIN($M3*Model!$A$14+$N3,$O3)*$P3,0)</f>
         <v>102.55</v>
       </c>
-      <c r="U3" s="32">
-        <f>MAX(MIN($L3*Model!$A$15+$M3,$N3)*$O3,0)</f>
+      <c r="V3" s="32">
+        <f>MAX(MIN($M3*Model!$A$15+$N3,$O3)*$P3,0)</f>
         <v>100.6</v>
       </c>
-      <c r="V3" s="32">
-        <f>MAX(MIN($L3*Model!$A$16+$M3,$N3)*$O3,0)</f>
+      <c r="W3" s="32">
+        <f>MAX(MIN($M3*Model!$A$16+$N3,$O3)*$P3,0)</f>
         <v>98</v>
       </c>
-      <c r="W3" s="32">
-        <f>MAX(MIN($L3*Model!$A$17+$M3,$N3)*$O3,0)</f>
+      <c r="X3" s="32">
+        <f>MAX(MIN($M3*Model!$A$17+$N3,$O3)*$P3,0)</f>
         <v>94.75</v>
       </c>
-      <c r="X3" s="32">
-        <f>MAX(MIN($L3*Model!$A$18+$M3,$N3)*$O3,0)</f>
+      <c r="Y3" s="32">
+        <f>MAX(MIN($M3*Model!$A$18+$N3,$O3)*$P3,0)</f>
         <v>90.85</v>
       </c>
-      <c r="Y3" s="32">
-        <f>MAX(MIN($L3*Model!$A$19+$M3,$N3)*$O3,0)</f>
+      <c r="Z3" s="32">
+        <f>MAX(MIN($M3*Model!$A$19+$N3,$O3)*$P3,0)</f>
         <v>104</v>
       </c>
-      <c r="Z3" s="32">
-        <f>S3*Model!$B$13+T3*Model!$B$14+U3*Model!$B$15+V3*Model!$B$16+W3*Model!$B$17+X3*Model!$B$18+Y3*Model!$B$19</f>
+      <c r="AA3" s="32">
+        <f>T3*Model!$B$13+U3*Model!$B$14+V3*Model!$B$15+W3*Model!$B$16+X3*Model!$B$17+Y3*Model!$B$18+Z3*Model!$B$19</f>
         <v>97.48</v>
       </c>
-      <c r="AA3" s="33">
+      <c r="AB3" s="33">
         <v>0.3</v>
       </c>
-      <c r="AB3" s="33">
+      <c r="AC3" s="33">
         <v>1.2</v>
       </c>
-      <c r="AC3" s="31" t="str">
-        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AD3,";",'7.62x51-ammo'!$AE3,";",'7.62x51-ammo'!$AF3,";",'7.62x51-ammo'!$AG3,")")</f>
+      <c r="AD3" s="31" t="str">
+        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AE3,";",'7.62x51-ammo'!$AF3,";",'7.62x51-ammo'!$AG3,";",'7.62x51-ammo'!$AH3,")")</f>
         <v>stat(bullet_velocity;0.6;1.1;1500;3000)</v>
       </c>
-      <c r="AD3" s="34">
+      <c r="AE3" s="34">
         <v>0.6</v>
       </c>
-      <c r="AE3" s="34">
+      <c r="AF3" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="AF3" s="35">
+      <c r="AG3" s="35">
         <v>1500</v>
       </c>
-      <c r="AG3" s="35">
+      <c r="AH3" s="35">
         <v>3000</v>
       </c>
-      <c r="AH3" s="36">
+      <c r="AI3" s="36">
         <f>Model!$B$4+IF(I3="",0,I3)</f>
         <v>2070</v>
       </c>
-      <c r="AI3" s="32">
-        <f t="shared" ref="AI3:AI11" si="0">MAX(AD3,MIN(AE3,AD3+(AH3-AF3)*(AE3-AD3)/(AG3-AF3)))</f>
+      <c r="AJ3" s="32">
+        <f t="shared" ref="AJ3:AJ11" si="0">MAX(AE3,MIN(AF3,AE3+(AI3-AG3)*(AF3-AE3)/(AH3-AG3)))</f>
         <v>0.79</v>
       </c>
-      <c r="AJ3" s="37">
+      <c r="AK3" s="37">
         <v>53</v>
       </c>
-      <c r="AK3" s="38" t="s">
+      <c r="AL3" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="AL3" s="39">
-        <f>C3*Model!$B$24+D3*Model!$B$25+E3*Model!$B$26+F3*Model!$B$27+G3*Model!$B$28+H3*Model!$B$29+I3*Model!$B$30+J3*Model!$B$31+K3*Model!$B$32</f>
+      <c r="AM3" s="39">
+        <f>C3*Model!$B$24+D3*Model!$B$25+E3*Model!$B$26+F3*Model!$B$27+G3*Model!$B$28+H3*Model!$B$29+I3*Model!$B$30+J3*Model!$B$31+K3*Model!$B$32+L3*Model!$B$33</f>
         <v>0</v>
       </c>
-      <c r="AM3" s="39">
-        <f>(Z3-Model!$B$5)*Model!$B$35</f>
+      <c r="AN3" s="39">
+        <f>(AA3-Model!$B$5)*Model!$B$36</f>
         <v>-3.779999999999994</v>
       </c>
-      <c r="AN3" s="39">
-        <f>(Model!$B$6-AA3)*Model!$B$36</f>
+      <c r="AO3" s="39">
+        <f>(Model!$B$6-AB3)*Model!$B$37</f>
         <v>9.9999999999999978E-2</v>
       </c>
-      <c r="AO3" s="39">
-        <f>(AB3-Model!$B$7)*Model!$B$37</f>
+      <c r="AP3" s="39">
+        <f>(AC3-Model!$B$7)*Model!$B$38</f>
         <v>1.0499999999999998</v>
       </c>
-      <c r="AP3" s="39">
-        <f>(AI3-Model!$B$8)*Model!$B$38</f>
+      <c r="AQ3" s="39">
+        <f>(AJ3-Model!$B$8)*Model!$B$39</f>
         <v>-0.83999999999999986</v>
       </c>
-      <c r="AQ3" s="39">
-        <f t="shared" ref="AQ3:AQ11" si="1">SUM(AL3:AP3)</f>
+      <c r="AR3" s="39">
+        <f t="shared" ref="AR3:AR11" si="1">SUM(AM3:AQ3)</f>
         <v>-3.469999999999994</v>
       </c>
     </row>
-    <row r="4" spans="1:43" ht="14.25" customHeight="1">
+    <row r="4" spans="1:44" ht="14.25" customHeight="1">
       <c r="A4" s="23" t="s">
         <v>101</v>
       </c>
@@ -1570,124 +1611,125 @@
         <v>0</v>
       </c>
       <c r="J4" s="28"/>
-      <c r="K4" s="29">
+      <c r="K4" s="28"/>
+      <c r="L4" s="29">
         <v>500</v>
       </c>
-      <c r="L4" s="30">
+      <c r="M4" s="30">
         <v>-2.8000000000000001E-2</v>
       </c>
-      <c r="M4" s="30">
+      <c r="N4" s="30">
         <v>104.5</v>
       </c>
-      <c r="N4" s="30">
+      <c r="O4" s="30">
         <v>104</v>
       </c>
-      <c r="O4" s="30">
+      <c r="P4" s="30">
         <v>1</v>
       </c>
-      <c r="P4" s="30">
+      <c r="Q4" s="30">
         <v>0.3</v>
       </c>
-      <c r="Q4" s="30">
+      <c r="R4" s="30">
         <v>0.5</v>
       </c>
-      <c r="R4" s="31">
+      <c r="S4" s="31">
         <v>2.5</v>
       </c>
-      <c r="S4" s="32">
-        <f>MAX(MIN($L4*Model!$A$13+$M4,$N4)*$O4,0)</f>
+      <c r="T4" s="32">
+        <f>MAX(MIN($M4*Model!$A$13+$N4,$O4)*$P4,0)</f>
         <v>103.8</v>
       </c>
-      <c r="T4" s="32">
-        <f>MAX(MIN($L4*Model!$A$14+$M4,$N4)*$O4,0)</f>
+      <c r="U4" s="32">
+        <f>MAX(MIN($M4*Model!$A$14+$N4,$O4)*$P4,0)</f>
         <v>102.4</v>
       </c>
-      <c r="U4" s="32">
-        <f>MAX(MIN($L4*Model!$A$15+$M4,$N4)*$O4,0)</f>
+      <c r="V4" s="32">
+        <f>MAX(MIN($M4*Model!$A$15+$N4,$O4)*$P4,0)</f>
         <v>100.3</v>
       </c>
-      <c r="V4" s="32">
-        <f>MAX(MIN($L4*Model!$A$16+$M4,$N4)*$O4,0)</f>
+      <c r="W4" s="32">
+        <f>MAX(MIN($M4*Model!$A$16+$N4,$O4)*$P4,0)</f>
         <v>97.5</v>
       </c>
-      <c r="W4" s="32">
-        <f>MAX(MIN($L4*Model!$A$17+$M4,$N4)*$O4,0)</f>
+      <c r="X4" s="32">
+        <f>MAX(MIN($M4*Model!$A$17+$N4,$O4)*$P4,0)</f>
         <v>94</v>
       </c>
-      <c r="X4" s="32">
-        <f>MAX(MIN($L4*Model!$A$18+$M4,$N4)*$O4,0)</f>
+      <c r="Y4" s="32">
+        <f>MAX(MIN($M4*Model!$A$18+$N4,$O4)*$P4,0)</f>
         <v>89.8</v>
       </c>
-      <c r="Y4" s="32">
-        <f>MAX(MIN($L4*Model!$A$19+$M4,$N4)*$O4,0)</f>
+      <c r="Z4" s="32">
+        <f>MAX(MIN($M4*Model!$A$19+$N4,$O4)*$P4,0)</f>
         <v>104</v>
       </c>
-      <c r="Z4" s="32">
-        <f>S4*Model!$B$13+T4*Model!$B$14+U4*Model!$B$15+V4*Model!$B$16+W4*Model!$B$17+X4*Model!$B$18+Y4*Model!$B$19</f>
+      <c r="AA4" s="32">
+        <f>T4*Model!$B$13+U4*Model!$B$14+V4*Model!$B$15+W4*Model!$B$16+X4*Model!$B$17+Y4*Model!$B$18+Z4*Model!$B$19</f>
         <v>96.94</v>
       </c>
-      <c r="AA4" s="33">
+      <c r="AB4" s="33">
         <v>0.35</v>
       </c>
-      <c r="AB4" s="33">
+      <c r="AC4" s="33">
         <v>1.35</v>
       </c>
-      <c r="AC4" s="31" t="str">
-        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AD4,";",'7.62x51-ammo'!$AE4,";",'7.62x51-ammo'!$AF4,";",'7.62x51-ammo'!$AG4,")")</f>
+      <c r="AD4" s="31" t="str">
+        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AE4,";",'7.62x51-ammo'!$AF4,";",'7.62x51-ammo'!$AG4,";",'7.62x51-ammo'!$AH4,")")</f>
         <v>stat(bullet_velocity;0.55;1.05;1500;3000)</v>
       </c>
-      <c r="AD4" s="34">
+      <c r="AE4" s="34">
         <v>0.55000000000000004</v>
       </c>
-      <c r="AE4" s="34">
+      <c r="AF4" s="34">
         <v>1.05</v>
       </c>
-      <c r="AF4" s="35">
+      <c r="AG4" s="35">
         <v>1500</v>
       </c>
-      <c r="AG4" s="35">
+      <c r="AH4" s="35">
         <v>3000</v>
       </c>
-      <c r="AH4" s="36">
+      <c r="AI4" s="36">
         <f>Model!$B$4+IF(I4="",0,I4)</f>
         <v>2070</v>
       </c>
-      <c r="AI4" s="32">
+      <c r="AJ4" s="32">
         <f t="shared" si="0"/>
         <v>0.74</v>
       </c>
-      <c r="AJ4" s="37">
+      <c r="AK4" s="37">
         <v>51</v>
       </c>
-      <c r="AK4" s="38" t="s">
+      <c r="AL4" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="AL4" s="39">
-        <f>C4*Model!$B$24+D4*Model!$B$25+E4*Model!$B$26+F4*Model!$B$27+G4*Model!$B$28+H4*Model!$B$29+I4*Model!$B$30+J4*Model!$B$31+K4*Model!$B$32</f>
+      <c r="AM4" s="39">
+        <f>C4*Model!$B$24+D4*Model!$B$25+E4*Model!$B$26+F4*Model!$B$27+G4*Model!$B$28+H4*Model!$B$29+I4*Model!$B$30+J4*Model!$B$31+K4*Model!$B$32+L4*Model!$B$33</f>
         <v>3.4000000000000004</v>
       </c>
-      <c r="AM4" s="39">
-        <f>(Z4-Model!$B$5)*Model!$B$35</f>
+      <c r="AN4" s="39">
+        <f>(AA4-Model!$B$5)*Model!$B$36</f>
         <v>-4.5900000000000034</v>
       </c>
-      <c r="AN4" s="39">
-        <f>(Model!$B$6-AA4)*Model!$B$36</f>
+      <c r="AO4" s="39">
+        <f>(Model!$B$6-AB4)*Model!$B$37</f>
         <v>0</v>
       </c>
-      <c r="AO4" s="39">
-        <f>(AB4-Model!$B$7)*Model!$B$37</f>
+      <c r="AP4" s="39">
+        <f>(AC4-Model!$B$7)*Model!$B$38</f>
         <v>1.5000000000000004</v>
       </c>
-      <c r="AP4" s="39">
-        <f>(AI4-Model!$B$8)*Model!$B$38</f>
+      <c r="AQ4" s="39">
+        <f>(AJ4-Model!$B$8)*Model!$B$39</f>
         <v>-1.04</v>
       </c>
-      <c r="AQ4" s="39">
+      <c r="AR4" s="39">
         <f t="shared" si="1"/>
         <v>-0.73000000000000265</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="14.25" customHeight="1">
+    <row r="5" spans="1:44" ht="14.25" customHeight="1">
       <c r="A5" s="23" t="s">
         <v>86</v>
       </c>
@@ -1714,124 +1756,125 @@
         <v>-50</v>
       </c>
       <c r="J5" s="28"/>
-      <c r="K5" s="29">
+      <c r="K5" s="28"/>
+      <c r="L5" s="29">
         <v>1000</v>
       </c>
-      <c r="L5" s="30">
+      <c r="M5" s="30">
         <v>-2.5999999999999999E-2</v>
-      </c>
-      <c r="M5" s="30">
-        <v>105.5</v>
       </c>
       <c r="N5" s="30">
         <v>105.5</v>
       </c>
       <c r="O5" s="30">
+        <v>105.5</v>
+      </c>
+      <c r="P5" s="30">
         <v>1</v>
       </c>
-      <c r="P5" s="30">
+      <c r="Q5" s="30">
         <v>0.3</v>
       </c>
-      <c r="Q5" s="30">
+      <c r="R5" s="30">
         <v>0.5</v>
       </c>
-      <c r="R5" s="31">
+      <c r="S5" s="31">
         <v>2.5</v>
       </c>
-      <c r="S5" s="32">
-        <f>MAX(MIN($L5*Model!$A$13+$M5,$N5)*$O5,0)</f>
+      <c r="T5" s="32">
+        <f>MAX(MIN($M5*Model!$A$13+$N5,$O5)*$P5,0)</f>
         <v>104.85</v>
       </c>
-      <c r="T5" s="32">
-        <f>MAX(MIN($L5*Model!$A$14+$M5,$N5)*$O5,0)</f>
+      <c r="U5" s="32">
+        <f>MAX(MIN($M5*Model!$A$14+$N5,$O5)*$P5,0)</f>
         <v>103.55</v>
       </c>
-      <c r="U5" s="32">
-        <f>MAX(MIN($L5*Model!$A$15+$M5,$N5)*$O5,0)</f>
+      <c r="V5" s="32">
+        <f>MAX(MIN($M5*Model!$A$15+$N5,$O5)*$P5,0)</f>
         <v>101.6</v>
       </c>
-      <c r="V5" s="32">
-        <f>MAX(MIN($L5*Model!$A$16+$M5,$N5)*$O5,0)</f>
+      <c r="W5" s="32">
+        <f>MAX(MIN($M5*Model!$A$16+$N5,$O5)*$P5,0)</f>
         <v>99</v>
       </c>
-      <c r="W5" s="32">
-        <f>MAX(MIN($L5*Model!$A$17+$M5,$N5)*$O5,0)</f>
+      <c r="X5" s="32">
+        <f>MAX(MIN($M5*Model!$A$17+$N5,$O5)*$P5,0)</f>
         <v>95.75</v>
       </c>
-      <c r="X5" s="32">
-        <f>MAX(MIN($L5*Model!$A$18+$M5,$N5)*$O5,0)</f>
+      <c r="Y5" s="32">
+        <f>MAX(MIN($M5*Model!$A$18+$N5,$O5)*$P5,0)</f>
         <v>91.85</v>
       </c>
-      <c r="Y5" s="32">
-        <f>MAX(MIN($L5*Model!$A$19+$M5,$N5)*$O5,0)</f>
+      <c r="Z5" s="32">
+        <f>MAX(MIN($M5*Model!$A$19+$N5,$O5)*$P5,0)</f>
         <v>105.5</v>
       </c>
-      <c r="Z5" s="32">
-        <f>S5*Model!$B$13+T5*Model!$B$14+U5*Model!$B$15+V5*Model!$B$16+W5*Model!$B$17+X5*Model!$B$18+Y5*Model!$B$19</f>
+      <c r="AA5" s="32">
+        <f>T5*Model!$B$13+U5*Model!$B$14+V5*Model!$B$15+W5*Model!$B$16+X5*Model!$B$17+Y5*Model!$B$18+Z5*Model!$B$19</f>
         <v>98.48</v>
       </c>
-      <c r="AA5" s="33">
+      <c r="AB5" s="33">
         <v>0.45</v>
       </c>
-      <c r="AB5" s="33">
+      <c r="AC5" s="33">
         <v>1.1000000000000001</v>
       </c>
-      <c r="AC5" s="31" t="str">
-        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AD5,";",'7.62x51-ammo'!$AE5,";",'7.62x51-ammo'!$AF5,";",'7.62x51-ammo'!$AG5,")")</f>
+      <c r="AD5" s="31" t="str">
+        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AE5,";",'7.62x51-ammo'!$AF5,";",'7.62x51-ammo'!$AG5,";",'7.62x51-ammo'!$AH5,")")</f>
         <v>stat(bullet_velocity;0.2;0.7;1500;3000)</v>
       </c>
-      <c r="AD5" s="34">
+      <c r="AE5" s="34">
         <v>0.2</v>
       </c>
-      <c r="AE5" s="34">
+      <c r="AF5" s="34">
         <v>0.7</v>
       </c>
-      <c r="AF5" s="35">
+      <c r="AG5" s="35">
         <v>1500</v>
       </c>
-      <c r="AG5" s="35">
+      <c r="AH5" s="35">
         <v>3000</v>
       </c>
-      <c r="AH5" s="36">
+      <c r="AI5" s="36">
         <f>Model!$B$4+IF(I5="",0,I5)</f>
         <v>2020</v>
       </c>
-      <c r="AI5" s="32">
+      <c r="AJ5" s="32">
         <f t="shared" si="0"/>
         <v>0.37333333333333329</v>
       </c>
-      <c r="AJ5" s="37">
+      <c r="AK5" s="37">
         <v>49</v>
       </c>
-      <c r="AK5" s="38" t="s">
+      <c r="AL5" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="AL5" s="39">
-        <f>C5*Model!$B$24+D5*Model!$B$25+E5*Model!$B$26+F5*Model!$B$27+G5*Model!$B$28+H5*Model!$B$29+I5*Model!$B$30+J5*Model!$B$31+K5*Model!$B$32</f>
+      <c r="AM5" s="39">
+        <f>C5*Model!$B$24+D5*Model!$B$25+E5*Model!$B$26+F5*Model!$B$27+G5*Model!$B$28+H5*Model!$B$29+I5*Model!$B$30+J5*Model!$B$31+K5*Model!$B$32+L5*Model!$B$33</f>
         <v>-2.5499999999999998</v>
       </c>
-      <c r="AM5" s="39">
-        <f>(Z5-Model!$B$5)*Model!$B$35</f>
+      <c r="AN5" s="39">
+        <f>(AA5-Model!$B$5)*Model!$B$36</f>
         <v>-2.279999999999994</v>
       </c>
-      <c r="AN5" s="39">
-        <f>(Model!$B$6-AA5)*Model!$B$36</f>
+      <c r="AO5" s="39">
+        <f>(Model!$B$6-AB5)*Model!$B$37</f>
         <v>-0.20000000000000007</v>
       </c>
-      <c r="AO5" s="39">
-        <f>(AB5-Model!$B$7)*Model!$B$37</f>
+      <c r="AP5" s="39">
+        <f>(AC5-Model!$B$7)*Model!$B$38</f>
         <v>0.75000000000000033</v>
       </c>
-      <c r="AP5" s="39">
-        <f>(AI5-Model!$B$8)*Model!$B$38</f>
+      <c r="AQ5" s="39">
+        <f>(AJ5-Model!$B$8)*Model!$B$39</f>
         <v>-2.5066666666666668</v>
       </c>
-      <c r="AQ5" s="39">
+      <c r="AR5" s="39">
         <f t="shared" si="1"/>
         <v>-6.7866666666666609</v>
       </c>
     </row>
-    <row r="6" spans="1:43" ht="14.25" customHeight="1">
+    <row r="6" spans="1:44" ht="14.25" customHeight="1">
       <c r="A6" s="23" t="s">
         <v>88</v>
       </c>
@@ -1858,124 +1901,125 @@
         <v>-150</v>
       </c>
       <c r="J6" s="28"/>
-      <c r="K6" s="29">
+      <c r="K6" s="28"/>
+      <c r="L6" s="29">
         <v>3000</v>
       </c>
-      <c r="L6" s="30">
+      <c r="M6" s="30">
         <v>-1.7999999999999999E-2</v>
-      </c>
-      <c r="M6" s="30">
-        <v>104</v>
       </c>
       <c r="N6" s="30">
         <v>104</v>
       </c>
       <c r="O6" s="30">
+        <v>104</v>
+      </c>
+      <c r="P6" s="30">
         <v>1</v>
       </c>
-      <c r="P6" s="30">
+      <c r="Q6" s="30">
         <v>0.3</v>
       </c>
-      <c r="Q6" s="30">
+      <c r="R6" s="30">
         <v>0.5</v>
       </c>
-      <c r="R6" s="31">
+      <c r="S6" s="31">
         <v>2.5</v>
       </c>
-      <c r="S6" s="32">
-        <f>MAX(MIN($L6*Model!$A$13+$M6,$N6)*$O6,0)</f>
+      <c r="T6" s="32">
+        <f>MAX(MIN($M6*Model!$A$13+$N6,$O6)*$P6,0)</f>
         <v>103.55</v>
       </c>
-      <c r="T6" s="32">
-        <f>MAX(MIN($L6*Model!$A$14+$M6,$N6)*$O6,0)</f>
+      <c r="U6" s="32">
+        <f>MAX(MIN($M6*Model!$A$14+$N6,$O6)*$P6,0)</f>
         <v>102.65</v>
       </c>
-      <c r="U6" s="32">
-        <f>MAX(MIN($L6*Model!$A$15+$M6,$N6)*$O6,0)</f>
+      <c r="V6" s="32">
+        <f>MAX(MIN($M6*Model!$A$15+$N6,$O6)*$P6,0)</f>
         <v>101.3</v>
       </c>
-      <c r="V6" s="32">
-        <f>MAX(MIN($L6*Model!$A$16+$M6,$N6)*$O6,0)</f>
+      <c r="W6" s="32">
+        <f>MAX(MIN($M6*Model!$A$16+$N6,$O6)*$P6,0)</f>
         <v>99.5</v>
       </c>
-      <c r="W6" s="32">
-        <f>MAX(MIN($L6*Model!$A$17+$M6,$N6)*$O6,0)</f>
+      <c r="X6" s="32">
+        <f>MAX(MIN($M6*Model!$A$17+$N6,$O6)*$P6,0)</f>
         <v>97.25</v>
       </c>
-      <c r="X6" s="32">
-        <f>MAX(MIN($L6*Model!$A$18+$M6,$N6)*$O6,0)</f>
+      <c r="Y6" s="32">
+        <f>MAX(MIN($M6*Model!$A$18+$N6,$O6)*$P6,0)</f>
         <v>94.55</v>
       </c>
-      <c r="Y6" s="32">
-        <f>MAX(MIN($L6*Model!$A$19+$M6,$N6)*$O6,0)</f>
+      <c r="Z6" s="32">
+        <f>MAX(MIN($M6*Model!$A$19+$N6,$O6)*$P6,0)</f>
         <v>104</v>
       </c>
-      <c r="Z6" s="32">
-        <f>S6*Model!$B$13+T6*Model!$B$14+U6*Model!$B$15+V6*Model!$B$16+W6*Model!$B$17+X6*Model!$B$18+Y6*Model!$B$19</f>
+      <c r="AA6" s="32">
+        <f>T6*Model!$B$13+U6*Model!$B$14+V6*Model!$B$15+W6*Model!$B$16+X6*Model!$B$17+Y6*Model!$B$18+Z6*Model!$B$19</f>
         <v>99.14</v>
       </c>
-      <c r="AA6" s="33">
+      <c r="AB6" s="33">
         <v>0.1</v>
       </c>
-      <c r="AB6" s="33">
+      <c r="AC6" s="33">
         <v>0.9</v>
       </c>
-      <c r="AC6" s="31" t="str">
-        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AD6,";",'7.62x51-ammo'!$AE6,";",'7.62x51-ammo'!$AF6,";",'7.62x51-ammo'!$AG6,")")</f>
+      <c r="AD6" s="31" t="str">
+        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AE6,";",'7.62x51-ammo'!$AF6,";",'7.62x51-ammo'!$AG6,";",'7.62x51-ammo'!$AH6,")")</f>
         <v>stat(bullet_velocity;0.05;0.55;1500;3000)</v>
       </c>
-      <c r="AD6" s="34">
+      <c r="AE6" s="34">
         <v>0.05</v>
       </c>
-      <c r="AE6" s="34">
+      <c r="AF6" s="34">
         <v>0.55000000000000004</v>
       </c>
-      <c r="AF6" s="35">
+      <c r="AG6" s="35">
         <v>1500</v>
       </c>
-      <c r="AG6" s="35">
+      <c r="AH6" s="35">
         <v>3000</v>
       </c>
-      <c r="AH6" s="36">
+      <c r="AI6" s="36">
         <f>Model!$B$4+IF(I6="",0,I6)</f>
         <v>1920</v>
       </c>
-      <c r="AI6" s="32">
+      <c r="AJ6" s="32">
         <f t="shared" si="0"/>
         <v>0.19</v>
       </c>
-      <c r="AJ6" s="37">
+      <c r="AK6" s="37">
         <v>52</v>
       </c>
-      <c r="AK6" s="38" t="s">
+      <c r="AL6" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="AL6" s="39">
-        <f>C6*Model!$B$24+D6*Model!$B$25+E6*Model!$B$26+F6*Model!$B$27+G6*Model!$B$28+H6*Model!$B$29+I6*Model!$B$30+J6*Model!$B$31+K6*Model!$B$32</f>
+      <c r="AM6" s="39">
+        <f>C6*Model!$B$24+D6*Model!$B$25+E6*Model!$B$26+F6*Model!$B$27+G6*Model!$B$28+H6*Model!$B$29+I6*Model!$B$30+J6*Model!$B$31+K6*Model!$B$32+L6*Model!$B$33</f>
         <v>-6.15</v>
       </c>
-      <c r="AM6" s="39">
-        <f>(Z6-Model!$B$5)*Model!$B$35</f>
+      <c r="AN6" s="39">
+        <f>(AA6-Model!$B$5)*Model!$B$36</f>
         <v>-1.2899999999999991</v>
       </c>
-      <c r="AN6" s="39">
-        <f>(Model!$B$6-AA6)*Model!$B$36</f>
+      <c r="AO6" s="39">
+        <f>(Model!$B$6-AB6)*Model!$B$37</f>
         <v>0.49999999999999994</v>
       </c>
-      <c r="AO6" s="39">
-        <f>(AB6-Model!$B$7)*Model!$B$37</f>
+      <c r="AP6" s="39">
+        <f>(AC6-Model!$B$7)*Model!$B$38</f>
         <v>0.15000000000000013</v>
       </c>
-      <c r="AP6" s="39">
-        <f>(AI6-Model!$B$8)*Model!$B$38</f>
+      <c r="AQ6" s="39">
+        <f>(AJ6-Model!$B$8)*Model!$B$39</f>
         <v>-3.24</v>
       </c>
-      <c r="AQ6" s="39">
+      <c r="AR6" s="39">
         <f t="shared" si="1"/>
         <v>-10.029999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:43" ht="14.25" customHeight="1">
+    <row r="7" spans="1:44" ht="14.25" customHeight="1">
       <c r="A7" s="23" t="s">
         <v>90</v>
       </c>
@@ -2002,124 +2046,125 @@
         <v>0</v>
       </c>
       <c r="J7" s="28"/>
-      <c r="K7" s="29">
+      <c r="K7" s="28"/>
+      <c r="L7" s="29">
         <v>2500</v>
       </c>
-      <c r="L7" s="30">
+      <c r="M7" s="30">
         <v>-2.1999999999999999E-2</v>
       </c>
-      <c r="M7" s="30">
+      <c r="N7" s="30">
         <v>104</v>
       </c>
-      <c r="N7" s="30">
+      <c r="O7" s="30">
         <v>103</v>
       </c>
-      <c r="O7" s="30">
+      <c r="P7" s="30">
         <v>1</v>
       </c>
-      <c r="P7" s="30">
+      <c r="Q7" s="30">
         <v>0.3</v>
       </c>
-      <c r="Q7" s="30">
+      <c r="R7" s="30">
         <v>0.5</v>
       </c>
-      <c r="R7" s="31">
+      <c r="S7" s="31">
         <v>2.5</v>
       </c>
-      <c r="S7" s="32">
-        <f>MAX(MIN($L7*Model!$A$13+$M7,$N7)*$O7,0)</f>
+      <c r="T7" s="32">
+        <f>MAX(MIN($M7*Model!$A$13+$N7,$O7)*$P7,0)</f>
         <v>103</v>
       </c>
-      <c r="T7" s="32">
-        <f>MAX(MIN($L7*Model!$A$14+$M7,$N7)*$O7,0)</f>
+      <c r="U7" s="32">
+        <f>MAX(MIN($M7*Model!$A$14+$N7,$O7)*$P7,0)</f>
         <v>102.35</v>
       </c>
-      <c r="U7" s="32">
-        <f>MAX(MIN($L7*Model!$A$15+$M7,$N7)*$O7,0)</f>
+      <c r="V7" s="32">
+        <f>MAX(MIN($M7*Model!$A$15+$N7,$O7)*$P7,0)</f>
         <v>100.7</v>
       </c>
-      <c r="V7" s="32">
-        <f>MAX(MIN($L7*Model!$A$16+$M7,$N7)*$O7,0)</f>
+      <c r="W7" s="32">
+        <f>MAX(MIN($M7*Model!$A$16+$N7,$O7)*$P7,0)</f>
         <v>98.5</v>
       </c>
-      <c r="W7" s="32">
-        <f>MAX(MIN($L7*Model!$A$17+$M7,$N7)*$O7,0)</f>
+      <c r="X7" s="32">
+        <f>MAX(MIN($M7*Model!$A$17+$N7,$O7)*$P7,0)</f>
         <v>95.75</v>
       </c>
-      <c r="X7" s="32">
-        <f>MAX(MIN($L7*Model!$A$18+$M7,$N7)*$O7,0)</f>
+      <c r="Y7" s="32">
+        <f>MAX(MIN($M7*Model!$A$18+$N7,$O7)*$P7,0)</f>
         <v>92.45</v>
       </c>
-      <c r="Y7" s="32">
-        <f>MAX(MIN($L7*Model!$A$19+$M7,$N7)*$O7,0)</f>
+      <c r="Z7" s="32">
+        <f>MAX(MIN($M7*Model!$A$19+$N7,$O7)*$P7,0)</f>
         <v>103</v>
       </c>
-      <c r="Z7" s="32">
-        <f>S7*Model!$B$13+T7*Model!$B$14+U7*Model!$B$15+V7*Model!$B$16+W7*Model!$B$17+X7*Model!$B$18+Y7*Model!$B$19</f>
+      <c r="AA7" s="32">
+        <f>T7*Model!$B$13+U7*Model!$B$14+V7*Model!$B$15+W7*Model!$B$16+X7*Model!$B$17+Y7*Model!$B$18+Z7*Model!$B$19</f>
         <v>98.015000000000015</v>
       </c>
-      <c r="AA7" s="33">
+      <c r="AB7" s="33">
         <v>0.15</v>
       </c>
-      <c r="AB7" s="33">
+      <c r="AC7" s="33">
         <v>1</v>
       </c>
-      <c r="AC7" s="31" t="str">
-        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AD7,";",'7.62x51-ammo'!$AE7,";",'7.62x51-ammo'!$AF7,";",'7.62x51-ammo'!$AG7,")")</f>
+      <c r="AD7" s="31" t="str">
+        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AE7,";",'7.62x51-ammo'!$AF7,";",'7.62x51-ammo'!$AG7,";",'7.62x51-ammo'!$AH7,")")</f>
         <v>stat(bullet_velocity;1.1;1.6;1500;3000)</v>
       </c>
-      <c r="AD7" s="34">
+      <c r="AE7" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="AE7" s="34">
+      <c r="AF7" s="34">
         <v>1.6</v>
       </c>
-      <c r="AF7" s="35">
+      <c r="AG7" s="35">
         <v>1500</v>
       </c>
-      <c r="AG7" s="35">
+      <c r="AH7" s="35">
         <v>3000</v>
       </c>
-      <c r="AH7" s="36">
+      <c r="AI7" s="36">
         <f>Model!$B$4+IF(I7="",0,I7)</f>
         <v>2070</v>
       </c>
-      <c r="AI7" s="32">
+      <c r="AJ7" s="32">
         <f t="shared" si="0"/>
         <v>1.29</v>
       </c>
-      <c r="AJ7" s="37">
+      <c r="AK7" s="37">
         <v>48</v>
       </c>
-      <c r="AK7" s="38" t="s">
+      <c r="AL7" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="AL7" s="39">
-        <f>C7*Model!$B$24+D7*Model!$B$25+E7*Model!$B$26+F7*Model!$B$27+G7*Model!$B$28+H7*Model!$B$29+I7*Model!$B$30+J7*Model!$B$31+K7*Model!$B$32</f>
+      <c r="AM7" s="39">
+        <f>C7*Model!$B$24+D7*Model!$B$25+E7*Model!$B$26+F7*Model!$B$27+G7*Model!$B$28+H7*Model!$B$29+I7*Model!$B$30+J7*Model!$B$31+K7*Model!$B$32+L7*Model!$B$33</f>
         <v>-2.8000000000000003</v>
       </c>
-      <c r="AM7" s="39">
-        <f>(Z7-Model!$B$5)*Model!$B$35</f>
+      <c r="AN7" s="39">
+        <f>(AA7-Model!$B$5)*Model!$B$36</f>
         <v>-2.9774999999999778</v>
       </c>
-      <c r="AN7" s="39">
-        <f>(Model!$B$6-AA7)*Model!$B$36</f>
+      <c r="AO7" s="39">
+        <f>(Model!$B$6-AB7)*Model!$B$37</f>
         <v>0.39999999999999997</v>
       </c>
-      <c r="AO7" s="39">
-        <f>(AB7-Model!$B$7)*Model!$B$37</f>
+      <c r="AP7" s="39">
+        <f>(AC7-Model!$B$7)*Model!$B$38</f>
         <v>0.45000000000000007</v>
       </c>
-      <c r="AP7" s="39">
-        <f>(AI7-Model!$B$8)*Model!$B$38</f>
+      <c r="AQ7" s="39">
+        <f>(AJ7-Model!$B$8)*Model!$B$39</f>
         <v>1.1600000000000001</v>
       </c>
-      <c r="AQ7" s="39">
+      <c r="AR7" s="39">
         <f t="shared" si="1"/>
         <v>-3.7674999999999779</v>
       </c>
     </row>
-    <row r="8" spans="1:43" ht="14.25" customHeight="1">
+    <row r="8" spans="1:44" ht="14.25" customHeight="1">
       <c r="A8" s="23" t="s">
         <v>92</v>
       </c>
@@ -2146,124 +2191,125 @@
         <v>150</v>
       </c>
       <c r="J8" s="28"/>
-      <c r="K8" s="29">
+      <c r="K8" s="28"/>
+      <c r="L8" s="29">
         <v>2500</v>
       </c>
-      <c r="L8" s="30">
+      <c r="M8" s="30">
         <v>-2.4E-2</v>
       </c>
-      <c r="M8" s="30">
+      <c r="N8" s="30">
         <v>104.5</v>
       </c>
-      <c r="N8" s="30">
+      <c r="O8" s="30">
         <v>104</v>
       </c>
-      <c r="O8" s="30">
+      <c r="P8" s="30">
         <v>1</v>
       </c>
-      <c r="P8" s="30">
+      <c r="Q8" s="30">
         <v>0.3</v>
       </c>
-      <c r="Q8" s="30">
+      <c r="R8" s="30">
         <v>0.5</v>
       </c>
-      <c r="R8" s="31">
+      <c r="S8" s="31">
         <v>2.5</v>
       </c>
-      <c r="S8" s="32">
-        <f>MAX(MIN($L8*Model!$A$13+$M8,$N8)*$O8,0)</f>
+      <c r="T8" s="32">
+        <f>MAX(MIN($M8*Model!$A$13+$N8,$O8)*$P8,0)</f>
         <v>103.9</v>
       </c>
-      <c r="T8" s="32">
-        <f>MAX(MIN($L8*Model!$A$14+$M8,$N8)*$O8,0)</f>
+      <c r="U8" s="32">
+        <f>MAX(MIN($M8*Model!$A$14+$N8,$O8)*$P8,0)</f>
         <v>102.7</v>
       </c>
-      <c r="U8" s="32">
-        <f>MAX(MIN($L8*Model!$A$15+$M8,$N8)*$O8,0)</f>
+      <c r="V8" s="32">
+        <f>MAX(MIN($M8*Model!$A$15+$N8,$O8)*$P8,0)</f>
         <v>100.9</v>
       </c>
-      <c r="V8" s="32">
-        <f>MAX(MIN($L8*Model!$A$16+$M8,$N8)*$O8,0)</f>
+      <c r="W8" s="32">
+        <f>MAX(MIN($M8*Model!$A$16+$N8,$O8)*$P8,0)</f>
         <v>98.5</v>
       </c>
-      <c r="W8" s="32">
-        <f>MAX(MIN($L8*Model!$A$17+$M8,$N8)*$O8,0)</f>
+      <c r="X8" s="32">
+        <f>MAX(MIN($M8*Model!$A$17+$N8,$O8)*$P8,0)</f>
         <v>95.5</v>
       </c>
-      <c r="X8" s="32">
-        <f>MAX(MIN($L8*Model!$A$18+$M8,$N8)*$O8,0)</f>
+      <c r="Y8" s="32">
+        <f>MAX(MIN($M8*Model!$A$18+$N8,$O8)*$P8,0)</f>
         <v>91.9</v>
       </c>
-      <c r="Y8" s="32">
-        <f>MAX(MIN($L8*Model!$A$19+$M8,$N8)*$O8,0)</f>
+      <c r="Z8" s="32">
+        <f>MAX(MIN($M8*Model!$A$19+$N8,$O8)*$P8,0)</f>
         <v>104</v>
       </c>
-      <c r="Z8" s="32">
-        <f>S8*Model!$B$13+T8*Model!$B$14+U8*Model!$B$15+V8*Model!$B$16+W8*Model!$B$17+X8*Model!$B$18+Y8*Model!$B$19</f>
+      <c r="AA8" s="32">
+        <f>T8*Model!$B$13+U8*Model!$B$14+V8*Model!$B$15+W8*Model!$B$16+X8*Model!$B$17+Y8*Model!$B$18+Z8*Model!$B$19</f>
         <v>98.02000000000001</v>
       </c>
-      <c r="AA8" s="33">
+      <c r="AB8" s="33">
         <v>0.2</v>
       </c>
-      <c r="AB8" s="33">
+      <c r="AC8" s="33">
         <v>0.9</v>
       </c>
-      <c r="AC8" s="31" t="str">
-        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AD8,";",'7.62x51-ammo'!$AE8,";",'7.62x51-ammo'!$AF8,";",'7.62x51-ammo'!$AG8,")")</f>
+      <c r="AD8" s="31" t="str">
+        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AE8,";",'7.62x51-ammo'!$AF8,";",'7.62x51-ammo'!$AG8,";",'7.62x51-ammo'!$AH8,")")</f>
         <v>stat(bullet_velocity;0.85;1.35;1500;3000)</v>
       </c>
-      <c r="AD8" s="34">
+      <c r="AE8" s="34">
         <v>0.85</v>
       </c>
-      <c r="AE8" s="34">
+      <c r="AF8" s="34">
         <v>1.35</v>
       </c>
-      <c r="AF8" s="35">
+      <c r="AG8" s="35">
         <v>1500</v>
       </c>
-      <c r="AG8" s="35">
+      <c r="AH8" s="35">
         <v>3000</v>
       </c>
-      <c r="AH8" s="36">
+      <c r="AI8" s="36">
         <f>Model!$B$4+IF(I8="",0,I8)</f>
         <v>2220</v>
       </c>
-      <c r="AI8" s="32">
+      <c r="AJ8" s="32">
         <f t="shared" si="0"/>
         <v>1.0900000000000001</v>
       </c>
-      <c r="AJ8" s="37">
+      <c r="AK8" s="37">
         <v>47</v>
       </c>
-      <c r="AK8" s="38" t="s">
+      <c r="AL8" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="AL8" s="39">
-        <f>C8*Model!$B$24+D8*Model!$B$25+E8*Model!$B$26+F8*Model!$B$27+G8*Model!$B$28+H8*Model!$B$29+I8*Model!$B$30+J8*Model!$B$31+K8*Model!$B$32</f>
+      <c r="AM8" s="39">
+        <f>C8*Model!$B$24+D8*Model!$B$25+E8*Model!$B$26+F8*Model!$B$27+G8*Model!$B$28+H8*Model!$B$29+I8*Model!$B$30+J8*Model!$B$31+K8*Model!$B$32+L8*Model!$B$33</f>
         <v>-0.45000000000000018</v>
       </c>
-      <c r="AM8" s="39">
-        <f>(Z8-Model!$B$5)*Model!$B$35</f>
+      <c r="AN8" s="39">
+        <f>(AA8-Model!$B$5)*Model!$B$36</f>
         <v>-2.9699999999999847</v>
       </c>
-      <c r="AN8" s="39">
-        <f>(Model!$B$6-AA8)*Model!$B$36</f>
+      <c r="AO8" s="39">
+        <f>(Model!$B$6-AB8)*Model!$B$37</f>
         <v>0.29999999999999993</v>
       </c>
-      <c r="AO8" s="39">
-        <f>(AB8-Model!$B$7)*Model!$B$37</f>
+      <c r="AP8" s="39">
+        <f>(AC8-Model!$B$7)*Model!$B$38</f>
         <v>0.15000000000000013</v>
       </c>
-      <c r="AP8" s="39">
-        <f>(AI8-Model!$B$8)*Model!$B$38</f>
+      <c r="AQ8" s="39">
+        <f>(AJ8-Model!$B$8)*Model!$B$39</f>
         <v>0.36000000000000032</v>
       </c>
-      <c r="AQ8" s="39">
+      <c r="AR8" s="39">
         <f t="shared" si="1"/>
         <v>-2.6099999999999843</v>
       </c>
     </row>
-    <row r="9" spans="1:43" ht="14.25" customHeight="1">
+    <row r="9" spans="1:44" ht="14.25" customHeight="1">
       <c r="A9" s="23" t="s">
         <v>94</v>
       </c>
@@ -2290,124 +2336,125 @@
         <v>150</v>
       </c>
       <c r="J9" s="26"/>
-      <c r="K9" s="29">
+      <c r="K9" s="26"/>
+      <c r="L9" s="29">
         <v>4000</v>
       </c>
-      <c r="L9" s="30">
+      <c r="M9" s="30">
         <v>-0.02</v>
       </c>
-      <c r="M9" s="30">
+      <c r="N9" s="30">
         <v>103</v>
       </c>
-      <c r="N9" s="30">
+      <c r="O9" s="30">
         <v>102</v>
       </c>
-      <c r="O9" s="30">
+      <c r="P9" s="30">
         <v>1</v>
       </c>
-      <c r="P9" s="30">
+      <c r="Q9" s="30">
         <v>0.25</v>
       </c>
-      <c r="Q9" s="30">
+      <c r="R9" s="30">
         <v>0.45</v>
       </c>
-      <c r="R9" s="41">
+      <c r="S9" s="41">
         <v>2.5</v>
       </c>
-      <c r="S9" s="42">
-        <f>MAX(MIN($L9*Model!$A$13+$M9,$N9)*$O9,0)</f>
+      <c r="T9" s="42">
+        <f>MAX(MIN($M9*Model!$A$13+$N9,$O9)*$P9,0)</f>
         <v>102</v>
       </c>
-      <c r="T9" s="42">
-        <f>MAX(MIN($L9*Model!$A$14+$M9,$N9)*$O9,0)</f>
+      <c r="U9" s="42">
+        <f>MAX(MIN($M9*Model!$A$14+$N9,$O9)*$P9,0)</f>
         <v>101.5</v>
       </c>
-      <c r="U9" s="42">
-        <f>MAX(MIN($L9*Model!$A$15+$M9,$N9)*$O9,0)</f>
+      <c r="V9" s="42">
+        <f>MAX(MIN($M9*Model!$A$15+$N9,$O9)*$P9,0)</f>
         <v>100</v>
       </c>
-      <c r="V9" s="42">
-        <f>MAX(MIN($L9*Model!$A$16+$M9,$N9)*$O9,0)</f>
+      <c r="W9" s="42">
+        <f>MAX(MIN($M9*Model!$A$16+$N9,$O9)*$P9,0)</f>
         <v>98</v>
       </c>
-      <c r="W9" s="42">
-        <f>MAX(MIN($L9*Model!$A$17+$M9,$N9)*$O9,0)</f>
+      <c r="X9" s="42">
+        <f>MAX(MIN($M9*Model!$A$17+$N9,$O9)*$P9,0)</f>
         <v>95.5</v>
       </c>
-      <c r="X9" s="42">
-        <f>MAX(MIN($L9*Model!$A$18+$M9,$N9)*$O9,0)</f>
+      <c r="Y9" s="42">
+        <f>MAX(MIN($M9*Model!$A$18+$N9,$O9)*$P9,0)</f>
         <v>92.5</v>
       </c>
-      <c r="Y9" s="42">
-        <f>MAX(MIN($L9*Model!$A$19+$M9,$N9)*$O9,0)</f>
+      <c r="Z9" s="42">
+        <f>MAX(MIN($M9*Model!$A$19+$N9,$O9)*$P9,0)</f>
         <v>102</v>
       </c>
-      <c r="Z9" s="42">
-        <f>S9*Model!$B$13+T9*Model!$B$14+U9*Model!$B$15+V9*Model!$B$16+W9*Model!$B$17+X9*Model!$B$18+Y9*Model!$B$19</f>
+      <c r="AA9" s="42">
+        <f>T9*Model!$B$13+U9*Model!$B$14+V9*Model!$B$15+W9*Model!$B$16+X9*Model!$B$17+Y9*Model!$B$18+Z9*Model!$B$19</f>
         <v>97.550000000000011</v>
       </c>
-      <c r="AA9" s="33">
+      <c r="AB9" s="33">
         <v>0.15</v>
       </c>
-      <c r="AB9" s="33">
+      <c r="AC9" s="33">
         <v>1</v>
       </c>
-      <c r="AC9" s="41" t="str">
-        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AD9,";",'7.62x51-ammo'!$AE9,";",'7.62x51-ammo'!$AF9,";",'7.62x51-ammo'!$AG9,")")</f>
+      <c r="AD9" s="41" t="str">
+        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AE9,";",'7.62x51-ammo'!$AF9,";",'7.62x51-ammo'!$AG9,";",'7.62x51-ammo'!$AH9,")")</f>
         <v>stat(bullet_velocity;1.5;2;1500;3000)</v>
       </c>
-      <c r="AD9" s="34">
+      <c r="AE9" s="34">
         <v>1.5</v>
       </c>
-      <c r="AE9" s="34">
+      <c r="AF9" s="34">
         <v>2</v>
       </c>
-      <c r="AF9" s="43">
+      <c r="AG9" s="43">
         <v>1500</v>
       </c>
-      <c r="AG9" s="43">
+      <c r="AH9" s="43">
         <v>3000</v>
       </c>
-      <c r="AH9" s="44">
+      <c r="AI9" s="44">
         <f>Model!$B$4+IF(I9="",0,I9)</f>
         <v>2220</v>
       </c>
-      <c r="AI9" s="42">
+      <c r="AJ9" s="42">
         <f t="shared" si="0"/>
         <v>1.74</v>
       </c>
-      <c r="AJ9" s="37">
+      <c r="AK9" s="37">
         <v>50</v>
       </c>
-      <c r="AK9" s="45" t="s">
+      <c r="AL9" s="45" t="s">
         <v>84</v>
       </c>
-      <c r="AL9" s="46">
-        <f>C9*Model!$B$24+D9*Model!$B$25+E9*Model!$B$26+F9*Model!$B$27+G9*Model!$B$28+H9*Model!$B$29+I9*Model!$B$30+J9*Model!$B$31+K9*Model!$B$32</f>
+      <c r="AM9" s="39">
+        <f>C9*Model!$B$24+D9*Model!$B$25+E9*Model!$B$26+F9*Model!$B$27+G9*Model!$B$28+H9*Model!$B$29+I9*Model!$B$30+J9*Model!$B$31+K9*Model!$B$32+L9*Model!$B$33</f>
         <v>-1.9500000000000002</v>
       </c>
-      <c r="AM9" s="46">
-        <f>(Z9-Model!$B$5)*Model!$B$35</f>
+      <c r="AN9" s="46">
+        <f>(AA9-Model!$B$5)*Model!$B$36</f>
         <v>-3.6749999999999829</v>
       </c>
-      <c r="AN9" s="46">
-        <f>(Model!$B$6-AA9)*Model!$B$36</f>
+      <c r="AO9" s="46">
+        <f>(Model!$B$6-AB9)*Model!$B$37</f>
         <v>0.39999999999999997</v>
       </c>
-      <c r="AO9" s="46">
-        <f>(AB9-Model!$B$7)*Model!$B$37</f>
+      <c r="AP9" s="46">
+        <f>(AC9-Model!$B$7)*Model!$B$38</f>
         <v>0.45000000000000007</v>
       </c>
-      <c r="AP9" s="46">
-        <f>(AI9-Model!$B$8)*Model!$B$38</f>
+      <c r="AQ9" s="46">
+        <f>(AJ9-Model!$B$8)*Model!$B$39</f>
         <v>2.96</v>
       </c>
-      <c r="AQ9" s="46">
+      <c r="AR9" s="46">
         <f t="shared" si="1"/>
         <v>-1.8149999999999826</v>
       </c>
     </row>
-    <row r="10" spans="1:43" ht="14.25" customHeight="1">
+    <row r="10" spans="1:44" ht="14.25" customHeight="1">
       <c r="A10" s="23" t="s">
         <v>96</v>
       </c>
@@ -2434,124 +2481,125 @@
         <v>200</v>
       </c>
       <c r="J10" s="28"/>
-      <c r="K10" s="29">
+      <c r="K10" s="28"/>
+      <c r="L10" s="29">
         <v>3500</v>
       </c>
-      <c r="L10" s="30">
+      <c r="M10" s="30">
         <v>-3.2000000000000001E-2</v>
       </c>
-      <c r="M10" s="30">
+      <c r="N10" s="30">
         <v>106.5</v>
       </c>
-      <c r="N10" s="30">
+      <c r="O10" s="30">
         <v>106</v>
       </c>
-      <c r="O10" s="30">
+      <c r="P10" s="30">
         <v>1</v>
       </c>
-      <c r="P10" s="30">
+      <c r="Q10" s="30">
         <v>0.3</v>
       </c>
-      <c r="Q10" s="30">
+      <c r="R10" s="30">
         <v>0.5</v>
       </c>
-      <c r="R10" s="31">
+      <c r="S10" s="31">
         <v>2.5</v>
       </c>
-      <c r="S10" s="32">
-        <f>MAX(MIN($L10*Model!$A$13+$M10,$N10)*$O10,0)</f>
+      <c r="T10" s="32">
+        <f>MAX(MIN($M10*Model!$A$13+$N10,$O10)*$P10,0)</f>
         <v>105.7</v>
       </c>
-      <c r="T10" s="32">
-        <f>MAX(MIN($L10*Model!$A$14+$M10,$N10)*$O10,0)</f>
+      <c r="U10" s="32">
+        <f>MAX(MIN($M10*Model!$A$14+$N10,$O10)*$P10,0)</f>
         <v>104.1</v>
       </c>
-      <c r="U10" s="32">
-        <f>MAX(MIN($L10*Model!$A$15+$M10,$N10)*$O10,0)</f>
+      <c r="V10" s="32">
+        <f>MAX(MIN($M10*Model!$A$15+$N10,$O10)*$P10,0)</f>
         <v>101.7</v>
       </c>
-      <c r="V10" s="32">
-        <f>MAX(MIN($L10*Model!$A$16+$M10,$N10)*$O10,0)</f>
+      <c r="W10" s="32">
+        <f>MAX(MIN($M10*Model!$A$16+$N10,$O10)*$P10,0)</f>
         <v>98.5</v>
       </c>
-      <c r="W10" s="32">
-        <f>MAX(MIN($L10*Model!$A$17+$M10,$N10)*$O10,0)</f>
+      <c r="X10" s="32">
+        <f>MAX(MIN($M10*Model!$A$17+$N10,$O10)*$P10,0)</f>
         <v>94.5</v>
       </c>
-      <c r="X10" s="32">
-        <f>MAX(MIN($L10*Model!$A$18+$M10,$N10)*$O10,0)</f>
+      <c r="Y10" s="32">
+        <f>MAX(MIN($M10*Model!$A$18+$N10,$O10)*$P10,0)</f>
         <v>89.7</v>
       </c>
-      <c r="Y10" s="32">
-        <f>MAX(MIN($L10*Model!$A$19+$M10,$N10)*$O10,0)</f>
+      <c r="Z10" s="32">
+        <f>MAX(MIN($M10*Model!$A$19+$N10,$O10)*$P10,0)</f>
         <v>106</v>
       </c>
-      <c r="Z10" s="32">
-        <f>S10*Model!$B$13+T10*Model!$B$14+U10*Model!$B$15+V10*Model!$B$16+W10*Model!$B$17+X10*Model!$B$18+Y10*Model!$B$19</f>
+      <c r="AA10" s="32">
+        <f>T10*Model!$B$13+U10*Model!$B$14+V10*Model!$B$15+W10*Model!$B$16+X10*Model!$B$17+Y10*Model!$B$18+Z10*Model!$B$19</f>
         <v>97.860000000000014</v>
       </c>
-      <c r="AA10" s="33">
+      <c r="AB10" s="33">
         <v>0.3</v>
       </c>
-      <c r="AB10" s="33">
+      <c r="AC10" s="33">
         <v>0.8</v>
       </c>
-      <c r="AC10" s="31" t="str">
-        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AD10,";",'7.62x51-ammo'!$AE10,";",'7.62x51-ammo'!$AF10,";",'7.62x51-ammo'!$AG10,")")</f>
+      <c r="AD10" s="31" t="str">
+        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AE10,";",'7.62x51-ammo'!$AF10,";",'7.62x51-ammo'!$AG10,";",'7.62x51-ammo'!$AH10,")")</f>
         <v>stat(bullet_velocity;0.35;0.85;1500;3000)</v>
       </c>
-      <c r="AD10" s="34">
+      <c r="AE10" s="34">
         <v>0.35</v>
       </c>
-      <c r="AE10" s="34">
+      <c r="AF10" s="34">
         <v>0.85</v>
       </c>
-      <c r="AF10" s="35">
+      <c r="AG10" s="35">
         <v>1500</v>
       </c>
-      <c r="AG10" s="35">
+      <c r="AH10" s="35">
         <v>3000</v>
       </c>
-      <c r="AH10" s="36">
+      <c r="AI10" s="36">
         <f>Model!$B$4+IF(I10="",0,I10)</f>
         <v>2270</v>
       </c>
-      <c r="AI10" s="32">
+      <c r="AJ10" s="32">
         <f t="shared" si="0"/>
         <v>0.60666666666666669</v>
       </c>
-      <c r="AJ10" s="37">
+      <c r="AK10" s="37">
         <v>46</v>
       </c>
-      <c r="AK10" s="38" t="s">
+      <c r="AL10" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="AL10" s="39">
-        <f>C10*Model!$B$24+D10*Model!$B$25+E10*Model!$B$26+F10*Model!$B$27+G10*Model!$B$28+H10*Model!$B$29+I10*Model!$B$30+J10*Model!$B$31+K10*Model!$B$32</f>
+      <c r="AM10" s="39">
+        <f>C10*Model!$B$24+D10*Model!$B$25+E10*Model!$B$26+F10*Model!$B$27+G10*Model!$B$28+H10*Model!$B$29+I10*Model!$B$30+J10*Model!$B$31+K10*Model!$B$32+L10*Model!$B$33</f>
         <v>1.5</v>
       </c>
-      <c r="AM10" s="39">
-        <f>(Z10-Model!$B$5)*Model!$B$35</f>
+      <c r="AN10" s="39">
+        <f>(AA10-Model!$B$5)*Model!$B$36</f>
         <v>-3.2099999999999795</v>
       </c>
-      <c r="AN10" s="39">
-        <f>(Model!$B$6-AA10)*Model!$B$36</f>
+      <c r="AO10" s="39">
+        <f>(Model!$B$6-AB10)*Model!$B$37</f>
         <v>9.9999999999999978E-2</v>
       </c>
-      <c r="AO10" s="39">
-        <f>(AB10-Model!$B$7)*Model!$B$37</f>
+      <c r="AP10" s="39">
+        <f>(AC10-Model!$B$7)*Model!$B$38</f>
         <v>-0.1499999999999998</v>
       </c>
-      <c r="AP10" s="39">
-        <f>(AI10-Model!$B$8)*Model!$B$38</f>
+      <c r="AQ10" s="39">
+        <f>(AJ10-Model!$B$8)*Model!$B$39</f>
         <v>-1.5733333333333333</v>
       </c>
-      <c r="AQ10" s="39">
+      <c r="AR10" s="39">
         <f t="shared" si="1"/>
         <v>-3.3333333333333126</v>
       </c>
     </row>
-    <row r="11" spans="1:43" ht="14.25" customHeight="1">
+    <row r="11" spans="1:44" ht="14.25" customHeight="1">
       <c r="A11" s="23" t="s">
         <v>98</v>
       </c>
@@ -2580,124 +2628,127 @@
       <c r="J11" s="28">
         <v>-0.03</v>
       </c>
-      <c r="K11" s="29">
+      <c r="K11" s="28">
+        <v>-0.7</v>
+      </c>
+      <c r="L11" s="29">
         <v>2500</v>
       </c>
-      <c r="L11" s="30">
+      <c r="M11" s="30">
         <v>-6.4000000000000001E-2</v>
-      </c>
-      <c r="M11" s="30">
-        <v>109.5</v>
       </c>
       <c r="N11" s="30">
         <v>109.5</v>
       </c>
       <c r="O11" s="30">
+        <v>109.5</v>
+      </c>
+      <c r="P11" s="30">
         <v>1</v>
       </c>
-      <c r="P11" s="30">
+      <c r="Q11" s="30">
         <v>0.3</v>
       </c>
-      <c r="Q11" s="30">
+      <c r="R11" s="30">
         <v>0.5</v>
       </c>
-      <c r="R11" s="31">
+      <c r="S11" s="31">
         <v>2.5</v>
       </c>
-      <c r="S11" s="32">
-        <f>MAX(MIN($L11*Model!$A$13+$M11,$N11)*$O11,0)</f>
+      <c r="T11" s="32">
+        <f>MAX(MIN($M11*Model!$A$13+$N11,$O11)*$P11,0)</f>
         <v>107.9</v>
       </c>
-      <c r="T11" s="32">
-        <f>MAX(MIN($L11*Model!$A$14+$M11,$N11)*$O11,0)</f>
+      <c r="U11" s="32">
+        <f>MAX(MIN($M11*Model!$A$14+$N11,$O11)*$P11,0)</f>
         <v>104.7</v>
       </c>
-      <c r="U11" s="32">
-        <f>MAX(MIN($L11*Model!$A$15+$M11,$N11)*$O11,0)</f>
+      <c r="V11" s="32">
+        <f>MAX(MIN($M11*Model!$A$15+$N11,$O11)*$P11,0)</f>
         <v>99.9</v>
       </c>
-      <c r="V11" s="32">
-        <f>MAX(MIN($L11*Model!$A$16+$M11,$N11)*$O11,0)</f>
+      <c r="W11" s="32">
+        <f>MAX(MIN($M11*Model!$A$16+$N11,$O11)*$P11,0)</f>
         <v>93.5</v>
       </c>
-      <c r="W11" s="32">
-        <f>MAX(MIN($L11*Model!$A$17+$M11,$N11)*$O11,0)</f>
+      <c r="X11" s="32">
+        <f>MAX(MIN($M11*Model!$A$17+$N11,$O11)*$P11,0)</f>
         <v>85.5</v>
       </c>
-      <c r="X11" s="32">
-        <f>MAX(MIN($L11*Model!$A$18+$M11,$N11)*$O11,0)</f>
+      <c r="Y11" s="32">
+        <f>MAX(MIN($M11*Model!$A$18+$N11,$O11)*$P11,0)</f>
         <v>75.900000000000006</v>
       </c>
-      <c r="Y11" s="32">
-        <f>MAX(MIN($L11*Model!$A$19+$M11,$N11)*$O11,0)</f>
+      <c r="Z11" s="32">
+        <f>MAX(MIN($M11*Model!$A$19+$N11,$O11)*$P11,0)</f>
         <v>109.5</v>
       </c>
-      <c r="Z11" s="32">
-        <f>S11*Model!$B$13+T11*Model!$B$14+U11*Model!$B$15+V11*Model!$B$16+W11*Model!$B$17+X11*Model!$B$18+Y11*Model!$B$19</f>
+      <c r="AA11" s="32">
+        <f>T11*Model!$B$13+U11*Model!$B$14+V11*Model!$B$15+W11*Model!$B$16+X11*Model!$B$17+Y11*Model!$B$18+Z11*Model!$B$19</f>
         <v>92.220000000000027</v>
       </c>
-      <c r="AA11" s="33">
+      <c r="AB11" s="33">
         <v>0.7</v>
       </c>
-      <c r="AB11" s="33">
+      <c r="AC11" s="33">
         <v>0.2</v>
       </c>
-      <c r="AC11" s="31" t="str">
-        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AD11,";",'7.62x51-ammo'!$AE11,";",'7.62x51-ammo'!$AF11,";",'7.62x51-ammo'!$AG11,")")</f>
+      <c r="AD11" s="31" t="str">
+        <f>CONCATENATE("stat(bullet_velocity;",'7.62x51-ammo'!$AE11,";",'7.62x51-ammo'!$AF11,";",'7.62x51-ammo'!$AG11,";",'7.62x51-ammo'!$AH11,")")</f>
         <v>stat(bullet_velocity;0.2;0.7;1500;3000)</v>
       </c>
-      <c r="AD11" s="34">
+      <c r="AE11" s="34">
         <v>0.2</v>
       </c>
-      <c r="AE11" s="34">
+      <c r="AF11" s="34">
         <v>0.7</v>
       </c>
-      <c r="AF11" s="35">
+      <c r="AG11" s="35">
         <v>1500</v>
       </c>
-      <c r="AG11" s="35">
+      <c r="AH11" s="35">
         <v>3000</v>
       </c>
-      <c r="AH11" s="36">
+      <c r="AI11" s="36">
         <f>Model!$B$4+IF(I11="",0,I11)</f>
         <v>1170</v>
       </c>
-      <c r="AI11" s="32">
+      <c r="AJ11" s="32">
         <f t="shared" si="0"/>
         <v>0.2</v>
       </c>
-      <c r="AJ11" s="37">
+      <c r="AK11" s="37">
         <v>45</v>
       </c>
-      <c r="AK11" s="38" t="s">
+      <c r="AL11" s="38" t="s">
         <v>84</v>
       </c>
-      <c r="AL11" s="39">
-        <f>C11*Model!$B$24+D11*Model!$B$25+E11*Model!$B$26+F11*Model!$B$27+G11*Model!$B$28+H11*Model!$B$29+I11*Model!$B$30+J11*Model!$B$31+K11*Model!$B$32</f>
-        <v>-1.8</v>
-      </c>
       <c r="AM11" s="39">
-        <f>(Z11-Model!$B$5)*Model!$B$35</f>
+        <f>C11*Model!$B$24+D11*Model!$B$25+E11*Model!$B$26+F11*Model!$B$27+G11*Model!$B$28+H11*Model!$B$29+I11*Model!$B$30+J11*Model!$B$31+K11*Model!$B$32+L11*Model!$B$33</f>
+        <v>5.2</v>
+      </c>
+      <c r="AN11" s="39">
+        <f>(AA11-Model!$B$5)*Model!$B$36</f>
         <v>-11.669999999999959</v>
       </c>
-      <c r="AN11" s="39">
-        <f>(Model!$B$6-AA11)*Model!$B$36</f>
+      <c r="AO11" s="39">
+        <f>(Model!$B$6-AB11)*Model!$B$37</f>
         <v>-0.7</v>
       </c>
-      <c r="AO11" s="39">
-        <f>(AB11-Model!$B$7)*Model!$B$37</f>
+      <c r="AP11" s="39">
+        <f>(AC11-Model!$B$7)*Model!$B$38</f>
         <v>-1.9499999999999997</v>
       </c>
-      <c r="AP11" s="39">
-        <f>(AI11-Model!$B$8)*Model!$B$38</f>
+      <c r="AQ11" s="39">
+        <f>(AJ11-Model!$B$8)*Model!$B$39</f>
         <v>-3.2</v>
       </c>
-      <c r="AQ11" s="39">
+      <c r="AR11" s="39">
         <f t="shared" si="1"/>
-        <v>-19.319999999999958</v>
-      </c>
-    </row>
-    <row r="12" spans="1:43" ht="14.25" customHeight="1">
+        <v>-12.319999999999958</v>
+      </c>
+    </row>
+    <row r="12" spans="1:44" ht="14.25" customHeight="1">
       <c r="A12" s="47"/>
       <c r="B12" s="48"/>
       <c r="C12" s="49"/>
@@ -2707,15 +2758,15 @@
       <c r="H12" s="51"/>
       <c r="I12" s="49"/>
       <c r="J12" s="50"/>
-      <c r="K12" s="52"/>
-      <c r="L12" s="53"/>
+      <c r="K12" s="50"/>
+      <c r="L12" s="52"/>
       <c r="M12" s="53"/>
       <c r="N12" s="53"/>
       <c r="O12" s="53"/>
       <c r="P12" s="53"/>
       <c r="Q12" s="53"/>
-      <c r="R12" s="52"/>
-      <c r="S12" s="50"/>
+      <c r="R12" s="53"/>
+      <c r="S12" s="52"/>
       <c r="T12" s="50"/>
       <c r="U12" s="50"/>
       <c r="V12" s="50"/>
@@ -2723,25 +2774,26 @@
       <c r="X12" s="50"/>
       <c r="Y12" s="50"/>
       <c r="Z12" s="50"/>
-      <c r="AA12" s="54"/>
+      <c r="AA12" s="50"/>
       <c r="AB12" s="54"/>
-      <c r="AC12" s="52"/>
-      <c r="AD12" s="50"/>
+      <c r="AC12" s="54"/>
+      <c r="AD12" s="52"/>
       <c r="AE12" s="50"/>
-      <c r="AF12" s="55"/>
+      <c r="AF12" s="50"/>
       <c r="AG12" s="55"/>
       <c r="AH12" s="55"/>
-      <c r="AI12" s="50"/>
-      <c r="AJ12" s="49"/>
-      <c r="AK12" s="52"/>
-      <c r="AL12" s="50"/>
+      <c r="AI12" s="55"/>
+      <c r="AJ12" s="50"/>
+      <c r="AK12" s="49"/>
+      <c r="AL12" s="52"/>
       <c r="AM12" s="50"/>
       <c r="AN12" s="50"/>
       <c r="AO12" s="50"/>
       <c r="AP12" s="50"/>
       <c r="AQ12" s="50"/>
-    </row>
-    <row r="13" spans="1:43" ht="14.25" customHeight="1">
+      <c r="AR12" s="50"/>
+    </row>
+    <row r="13" spans="1:44" ht="14.25" customHeight="1">
       <c r="A13" s="47"/>
       <c r="B13" s="48"/>
       <c r="C13" s="49"/>
@@ -2752,15 +2804,15 @@
       <c r="H13" s="51"/>
       <c r="I13" s="49"/>
       <c r="J13" s="50"/>
-      <c r="K13" s="52"/>
-      <c r="L13" s="53"/>
+      <c r="K13" s="50"/>
+      <c r="L13" s="52"/>
       <c r="M13" s="53"/>
       <c r="N13" s="53"/>
       <c r="O13" s="53"/>
       <c r="P13" s="53"/>
       <c r="Q13" s="53"/>
-      <c r="R13" s="52"/>
-      <c r="S13" s="50"/>
+      <c r="R13" s="53"/>
+      <c r="S13" s="52"/>
       <c r="T13" s="50"/>
       <c r="U13" s="50"/>
       <c r="V13" s="50"/>
@@ -2768,25 +2820,26 @@
       <c r="X13" s="50"/>
       <c r="Y13" s="50"/>
       <c r="Z13" s="50"/>
-      <c r="AA13" s="54"/>
+      <c r="AA13" s="50"/>
       <c r="AB13" s="54"/>
-      <c r="AC13" s="52"/>
-      <c r="AD13" s="50"/>
+      <c r="AC13" s="54"/>
+      <c r="AD13" s="52"/>
       <c r="AE13" s="50"/>
-      <c r="AF13" s="55"/>
+      <c r="AF13" s="50"/>
       <c r="AG13" s="55"/>
       <c r="AH13" s="55"/>
-      <c r="AI13" s="50"/>
-      <c r="AJ13" s="52"/>
+      <c r="AI13" s="55"/>
+      <c r="AJ13" s="50"/>
       <c r="AK13" s="52"/>
-      <c r="AL13" s="50"/>
+      <c r="AL13" s="52"/>
       <c r="AM13" s="50"/>
       <c r="AN13" s="50"/>
       <c r="AO13" s="50"/>
       <c r="AP13" s="50"/>
       <c r="AQ13" s="50"/>
-    </row>
-    <row r="14" spans="1:43" ht="14.25" customHeight="1">
+      <c r="AR13" s="50"/>
+    </row>
+    <row r="14" spans="1:44" ht="14.25" customHeight="1">
       <c r="A14" s="47"/>
       <c r="B14" s="48"/>
       <c r="C14" s="52"/>
@@ -2798,13 +2851,13 @@
       <c r="I14" s="52"/>
       <c r="J14" s="52"/>
       <c r="K14" s="52"/>
-      <c r="L14" s="53"/>
+      <c r="L14" s="52"/>
       <c r="M14" s="53"/>
       <c r="N14" s="53"/>
       <c r="O14" s="53"/>
       <c r="P14" s="53"/>
       <c r="Q14" s="53"/>
-      <c r="R14" s="52"/>
+      <c r="R14" s="53"/>
       <c r="S14" s="52"/>
       <c r="T14" s="52"/>
       <c r="U14" s="52"/>
@@ -2813,9 +2866,9 @@
       <c r="X14" s="52"/>
       <c r="Y14" s="52"/>
       <c r="Z14" s="52"/>
-      <c r="AA14" s="53"/>
+      <c r="AA14" s="52"/>
       <c r="AB14" s="53"/>
-      <c r="AC14" s="52"/>
+      <c r="AC14" s="53"/>
       <c r="AD14" s="52"/>
       <c r="AE14" s="52"/>
       <c r="AF14" s="52"/>
@@ -2830,8 +2883,9 @@
       <c r="AO14" s="52"/>
       <c r="AP14" s="52"/>
       <c r="AQ14" s="52"/>
-    </row>
-    <row r="15" spans="1:43" ht="14.25" customHeight="1">
+      <c r="AR14" s="52"/>
+    </row>
+    <row r="15" spans="1:44" ht="14.25" customHeight="1">
       <c r="A15" s="47"/>
       <c r="B15" s="48"/>
       <c r="C15" s="52"/>
@@ -2843,13 +2897,13 @@
       <c r="I15" s="52"/>
       <c r="J15" s="52"/>
       <c r="K15" s="52"/>
-      <c r="L15" s="53"/>
+      <c r="L15" s="52"/>
       <c r="M15" s="53"/>
       <c r="N15" s="53"/>
       <c r="O15" s="53"/>
       <c r="P15" s="53"/>
       <c r="Q15" s="53"/>
-      <c r="R15" s="52"/>
+      <c r="R15" s="53"/>
       <c r="S15" s="52"/>
       <c r="T15" s="52"/>
       <c r="U15" s="52"/>
@@ -2858,9 +2912,9 @@
       <c r="X15" s="52"/>
       <c r="Y15" s="52"/>
       <c r="Z15" s="52"/>
-      <c r="AA15" s="53"/>
+      <c r="AA15" s="52"/>
       <c r="AB15" s="53"/>
-      <c r="AC15" s="52"/>
+      <c r="AC15" s="53"/>
       <c r="AD15" s="52"/>
       <c r="AE15" s="52"/>
       <c r="AF15" s="52"/>
@@ -2875,8 +2929,9 @@
       <c r="AO15" s="52"/>
       <c r="AP15" s="52"/>
       <c r="AQ15" s="52"/>
-    </row>
-    <row r="16" spans="1:43" ht="14.25" customHeight="1">
+      <c r="AR15" s="52"/>
+    </row>
+    <row r="16" spans="1:44" ht="14.25" customHeight="1">
       <c r="A16" s="47"/>
       <c r="B16" s="48"/>
       <c r="C16" s="52"/>
@@ -2888,13 +2943,13 @@
       <c r="I16" s="52"/>
       <c r="J16" s="52"/>
       <c r="K16" s="52"/>
-      <c r="L16" s="53"/>
+      <c r="L16" s="52"/>
       <c r="M16" s="53"/>
       <c r="N16" s="53"/>
       <c r="O16" s="53"/>
       <c r="P16" s="53"/>
       <c r="Q16" s="53"/>
-      <c r="R16" s="52"/>
+      <c r="R16" s="53"/>
       <c r="S16" s="52"/>
       <c r="T16" s="52"/>
       <c r="U16" s="52"/>
@@ -2903,9 +2958,9 @@
       <c r="X16" s="52"/>
       <c r="Y16" s="52"/>
       <c r="Z16" s="52"/>
-      <c r="AA16" s="53"/>
+      <c r="AA16" s="52"/>
       <c r="AB16" s="53"/>
-      <c r="AC16" s="52"/>
+      <c r="AC16" s="53"/>
       <c r="AD16" s="52"/>
       <c r="AE16" s="52"/>
       <c r="AF16" s="52"/>
@@ -2920,8 +2975,9 @@
       <c r="AO16" s="52"/>
       <c r="AP16" s="52"/>
       <c r="AQ16" s="52"/>
-    </row>
-    <row r="17" spans="1:43" ht="14.25" customHeight="1">
+      <c r="AR16" s="52"/>
+    </row>
+    <row r="17" spans="1:44" ht="14.25" customHeight="1">
       <c r="A17" s="47"/>
       <c r="B17" s="48"/>
       <c r="C17" s="52"/>
@@ -2933,13 +2989,13 @@
       <c r="I17" s="52"/>
       <c r="J17" s="52"/>
       <c r="K17" s="52"/>
-      <c r="L17" s="53"/>
+      <c r="L17" s="52"/>
       <c r="M17" s="53"/>
       <c r="N17" s="53"/>
       <c r="O17" s="53"/>
       <c r="P17" s="53"/>
       <c r="Q17" s="53"/>
-      <c r="R17" s="52"/>
+      <c r="R17" s="53"/>
       <c r="S17" s="52"/>
       <c r="T17" s="52"/>
       <c r="U17" s="52"/>
@@ -2948,9 +3004,9 @@
       <c r="X17" s="52"/>
       <c r="Y17" s="52"/>
       <c r="Z17" s="52"/>
-      <c r="AA17" s="53"/>
-      <c r="AB17" s="56"/>
-      <c r="AC17" s="52"/>
+      <c r="AA17" s="52"/>
+      <c r="AB17" s="53"/>
+      <c r="AC17" s="56"/>
       <c r="AD17" s="52"/>
       <c r="AE17" s="52"/>
       <c r="AF17" s="52"/>
@@ -2965,8 +3021,9 @@
       <c r="AO17" s="52"/>
       <c r="AP17" s="52"/>
       <c r="AQ17" s="52"/>
-    </row>
-    <row r="18" spans="1:43" ht="14.25" customHeight="1">
+      <c r="AR17" s="52"/>
+    </row>
+    <row r="18" spans="1:44" ht="14.25" customHeight="1">
       <c r="A18" s="47"/>
       <c r="B18" s="48"/>
       <c r="C18" s="52"/>
@@ -2978,13 +3035,13 @@
       <c r="I18" s="52"/>
       <c r="J18" s="52"/>
       <c r="K18" s="52"/>
-      <c r="L18" s="53"/>
+      <c r="L18" s="52"/>
       <c r="M18" s="53"/>
       <c r="N18" s="53"/>
       <c r="O18" s="53"/>
       <c r="P18" s="53"/>
       <c r="Q18" s="53"/>
-      <c r="R18" s="52"/>
+      <c r="R18" s="53"/>
       <c r="S18" s="52"/>
       <c r="T18" s="52"/>
       <c r="U18" s="52"/>
@@ -2993,9 +3050,9 @@
       <c r="X18" s="52"/>
       <c r="Y18" s="52"/>
       <c r="Z18" s="52"/>
-      <c r="AA18" s="53"/>
-      <c r="AB18" s="56"/>
-      <c r="AC18" s="52"/>
+      <c r="AA18" s="52"/>
+      <c r="AB18" s="53"/>
+      <c r="AC18" s="56"/>
       <c r="AD18" s="52"/>
       <c r="AE18" s="52"/>
       <c r="AF18" s="52"/>
@@ -3010,8 +3067,9 @@
       <c r="AO18" s="52"/>
       <c r="AP18" s="52"/>
       <c r="AQ18" s="52"/>
-    </row>
-    <row r="19" spans="1:43" ht="14.25" customHeight="1">
+      <c r="AR18" s="52"/>
+    </row>
+    <row r="19" spans="1:44" ht="14.25" customHeight="1">
       <c r="A19" s="47"/>
       <c r="B19" s="48"/>
       <c r="C19" s="52"/>
@@ -3023,13 +3081,13 @@
       <c r="I19" s="52"/>
       <c r="J19" s="52"/>
       <c r="K19" s="52"/>
-      <c r="L19" s="53"/>
+      <c r="L19" s="52"/>
       <c r="M19" s="53"/>
       <c r="N19" s="53"/>
       <c r="O19" s="53"/>
       <c r="P19" s="53"/>
       <c r="Q19" s="53"/>
-      <c r="R19" s="52"/>
+      <c r="R19" s="53"/>
       <c r="S19" s="52"/>
       <c r="T19" s="52"/>
       <c r="U19" s="52"/>
@@ -3038,9 +3096,9 @@
       <c r="X19" s="52"/>
       <c r="Y19" s="52"/>
       <c r="Z19" s="52"/>
-      <c r="AA19" s="53"/>
-      <c r="AB19" s="56"/>
-      <c r="AC19" s="52"/>
+      <c r="AA19" s="52"/>
+      <c r="AB19" s="53"/>
+      <c r="AC19" s="56"/>
       <c r="AD19" s="52"/>
       <c r="AE19" s="52"/>
       <c r="AF19" s="52"/>
@@ -3055,8 +3113,9 @@
       <c r="AO19" s="52"/>
       <c r="AP19" s="52"/>
       <c r="AQ19" s="52"/>
-    </row>
-    <row r="20" spans="1:43" ht="14.25" customHeight="1">
+      <c r="AR19" s="52"/>
+    </row>
+    <row r="20" spans="1:44" ht="14.25" customHeight="1">
       <c r="A20" s="47"/>
       <c r="B20" s="48"/>
       <c r="C20" s="52"/>
@@ -3068,13 +3127,13 @@
       <c r="I20" s="52"/>
       <c r="J20" s="52"/>
       <c r="K20" s="52"/>
-      <c r="L20" s="53"/>
+      <c r="L20" s="52"/>
       <c r="M20" s="53"/>
       <c r="N20" s="53"/>
       <c r="O20" s="53"/>
       <c r="P20" s="53"/>
       <c r="Q20" s="53"/>
-      <c r="R20" s="52"/>
+      <c r="R20" s="53"/>
       <c r="S20" s="52"/>
       <c r="T20" s="52"/>
       <c r="U20" s="52"/>
@@ -3083,9 +3142,9 @@
       <c r="X20" s="52"/>
       <c r="Y20" s="52"/>
       <c r="Z20" s="52"/>
-      <c r="AA20" s="53"/>
-      <c r="AB20" s="56"/>
-      <c r="AC20" s="52"/>
+      <c r="AA20" s="52"/>
+      <c r="AB20" s="53"/>
+      <c r="AC20" s="56"/>
       <c r="AD20" s="52"/>
       <c r="AE20" s="52"/>
       <c r="AF20" s="52"/>
@@ -3100,8 +3159,9 @@
       <c r="AO20" s="52"/>
       <c r="AP20" s="52"/>
       <c r="AQ20" s="52"/>
-    </row>
-    <row r="21" spans="1:43" ht="14.25" customHeight="1">
+      <c r="AR20" s="52"/>
+    </row>
+    <row r="21" spans="1:44" ht="14.25" customHeight="1">
       <c r="A21" s="47"/>
       <c r="B21" s="48"/>
       <c r="C21" s="52"/>
@@ -3113,13 +3173,13 @@
       <c r="I21" s="52"/>
       <c r="J21" s="52"/>
       <c r="K21" s="52"/>
-      <c r="L21" s="53"/>
+      <c r="L21" s="52"/>
       <c r="M21" s="53"/>
       <c r="N21" s="53"/>
       <c r="O21" s="53"/>
       <c r="P21" s="53"/>
       <c r="Q21" s="53"/>
-      <c r="R21" s="52"/>
+      <c r="R21" s="53"/>
       <c r="S21" s="52"/>
       <c r="T21" s="52"/>
       <c r="U21" s="52"/>
@@ -3128,9 +3188,9 @@
       <c r="X21" s="52"/>
       <c r="Y21" s="52"/>
       <c r="Z21" s="52"/>
-      <c r="AA21" s="53"/>
-      <c r="AB21" s="56"/>
-      <c r="AC21" s="52"/>
+      <c r="AA21" s="52"/>
+      <c r="AB21" s="53"/>
+      <c r="AC21" s="56"/>
       <c r="AD21" s="52"/>
       <c r="AE21" s="52"/>
       <c r="AF21" s="52"/>
@@ -3145,18 +3205,19 @@
       <c r="AO21" s="52"/>
       <c r="AP21" s="52"/>
       <c r="AQ21" s="52"/>
-    </row>
-    <row r="22" spans="1:43" ht="14.25" customHeight="1"/>
-    <row r="23" spans="1:43" ht="14.25" customHeight="1"/>
-    <row r="24" spans="1:43" ht="14.25" customHeight="1"/>
-    <row r="25" spans="1:43" ht="14.25" customHeight="1"/>
-    <row r="26" spans="1:43" ht="14.25" customHeight="1"/>
-    <row r="27" spans="1:43" ht="14.25" customHeight="1"/>
-    <row r="28" spans="1:43" ht="14.25" customHeight="1"/>
-    <row r="29" spans="1:43" ht="14.25" customHeight="1"/>
-    <row r="30" spans="1:43" ht="14.25" customHeight="1"/>
-    <row r="31" spans="1:43" ht="14.25" customHeight="1"/>
-    <row r="32" spans="1:43" ht="14.25" customHeight="1"/>
+      <c r="AR21" s="52"/>
+    </row>
+    <row r="22" spans="1:44" ht="14.25" customHeight="1"/>
+    <row r="23" spans="1:44" ht="14.25" customHeight="1"/>
+    <row r="24" spans="1:44" ht="14.25" customHeight="1"/>
+    <row r="25" spans="1:44" ht="14.25" customHeight="1"/>
+    <row r="26" spans="1:44" ht="14.25" customHeight="1"/>
+    <row r="27" spans="1:44" ht="14.25" customHeight="1"/>
+    <row r="28" spans="1:44" ht="14.25" customHeight="1"/>
+    <row r="29" spans="1:44" ht="14.25" customHeight="1"/>
+    <row r="30" spans="1:44" ht="14.25" customHeight="1"/>
+    <row r="31" spans="1:44" ht="14.25" customHeight="1"/>
+    <row r="32" spans="1:44" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
     <row r="35" ht="14.25" customHeight="1"/>
@@ -4125,15 +4186,15 @@
     <row r="998" ht="14.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="AJ1:AK1"/>
-    <mergeCell ref="AL1:AQ1"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="L1:O1"/>
-    <mergeCell ref="S1:Z1"/>
-    <mergeCell ref="AA1:AG1"/>
-    <mergeCell ref="AH1:AI1"/>
+    <mergeCell ref="AK1:AL1"/>
+    <mergeCell ref="AM1:AR1"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="M1:P1"/>
+    <mergeCell ref="T1:AA1"/>
+    <mergeCell ref="AB1:AH1"/>
+    <mergeCell ref="AI1:AJ1"/>
   </mergeCells>
-  <conditionalFormatting sqref="AQ3:AQ13">
+  <conditionalFormatting sqref="AR3:AR13">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -4156,7 +4217,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C1000"/>
+  <dimension ref="A1:C1001"/>
   <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -4169,8 +4230,8 @@
       <c r="A1" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="59"/>
-      <c r="C1" s="60"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="59"/>
     </row>
     <row r="2" spans="1:3" ht="14.25" customHeight="1">
       <c r="A2" s="1"/>
@@ -4454,9 +4515,9 @@
       <c r="B30" s="17">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="C30" s="12" t="e">
-        <f ca="1">_xludf.CONCAT("1 point per +", 1/B30)</f>
-        <v>#NAME?</v>
+      <c r="C30" s="12" t="str">
+        <f>CONCATENATE("1 point per +", 1/B30)</f>
+        <v>1 point per +200</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
@@ -4471,73 +4532,83 @@
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="71" t="s">
+        <v>102</v>
+      </c>
+      <c r="B32" s="72">
+        <v>-10</v>
+      </c>
+      <c r="C32" s="71" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A33" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B32" s="15">
+      <c r="B33" s="15">
         <v>0</v>
       </c>
-      <c r="C32" s="12" t="s">
+      <c r="C33" s="12" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A33" s="8"/>
-      <c r="B33" s="18"/>
-      <c r="C33" s="8"/>
-    </row>
     <row r="34" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A34" s="67" t="s">
+      <c r="A34" s="8"/>
+      <c r="B34" s="18"/>
+      <c r="C34" s="8"/>
+    </row>
+    <row r="35" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A35" s="67" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="68"/>
-      <c r="C34" s="69"/>
-    </row>
-    <row r="35" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A35" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="B35" s="20">
-        <v>1.5</v>
-      </c>
-      <c r="C35" s="19" t="s">
-        <v>66</v>
-      </c>
+      <c r="B35" s="68"/>
+      <c r="C35" s="69"/>
     </row>
     <row r="36" spans="1:3" ht="14.25" customHeight="1">
       <c r="A36" s="19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B36" s="20">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="14.25" customHeight="1">
       <c r="A37" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B37" s="20">
+        <v>2</v>
+      </c>
+      <c r="C37" s="19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A38" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="20">
+      <c r="B38" s="20">
         <v>3</v>
       </c>
-      <c r="C37" s="19" t="s">
+      <c r="C38" s="19" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A38" s="21" t="s">
+    <row r="39" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A39" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="B38" s="22">
+      <c r="B39" s="22">
         <v>4</v>
       </c>
-      <c r="C38" s="21" t="s">
+      <c r="C39" s="21" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="40" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="41" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="42" spans="1:3" ht="14.25" customHeight="1"/>
@@ -5499,12 +5570,13 @@
     <row r="998" ht="14.25" customHeight="1"/>
     <row r="999" ht="14.25" customHeight="1"/>
     <row r="1000" ht="14.25" customHeight="1"/>
+    <row r="1001" ht="14.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A22:C22"/>
-    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A35:C35"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>

<commit_message>
im dumb (fix ammo sheets) and make subs volume 0.6
</commit_message>
<xml_diff>
--- a/changes/308-ammo-super.xlsx
+++ b/changes/308-ammo-super.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9634F945-6EDF-425D-959F-1E17C4F27852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78595AF7-8C18-4DEF-A64A-4F7D23248581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="7.62x51-ammo" sheetId="1" r:id="rId1"/>
@@ -880,6 +880,10 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -891,6 +895,7 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -904,11 +909,6 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1246,64 +1246,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:44" ht="24" customHeight="1">
-      <c r="A1" s="62" t="s">
+      <c r="A1" s="64" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="61"/>
-      <c r="D1" s="61"/>
-      <c r="E1" s="61"/>
-      <c r="F1" s="61"/>
-      <c r="G1" s="61"/>
-      <c r="H1" s="61"/>
-      <c r="I1" s="61"/>
-      <c r="J1" s="61"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="63" t="s">
+      <c r="B1" s="63"/>
+      <c r="C1" s="63"/>
+      <c r="D1" s="63"/>
+      <c r="E1" s="63"/>
+      <c r="F1" s="63"/>
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="63"/>
+      <c r="K1" s="65"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="66" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="61"/>
-      <c r="O1" s="61"/>
-      <c r="P1" s="59"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="61"/>
       <c r="Q1" s="13"/>
       <c r="R1" s="13"/>
       <c r="S1" s="13"/>
-      <c r="T1" s="64" t="s">
+      <c r="T1" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="U1" s="61"/>
-      <c r="V1" s="61"/>
-      <c r="W1" s="61"/>
-      <c r="X1" s="61"/>
-      <c r="Y1" s="61"/>
-      <c r="Z1" s="61"/>
-      <c r="AA1" s="59"/>
-      <c r="AB1" s="63" t="s">
+      <c r="U1" s="63"/>
+      <c r="V1" s="63"/>
+      <c r="W1" s="63"/>
+      <c r="X1" s="63"/>
+      <c r="Y1" s="63"/>
+      <c r="Z1" s="63"/>
+      <c r="AA1" s="61"/>
+      <c r="AB1" s="66" t="s">
         <v>27</v>
       </c>
-      <c r="AC1" s="61"/>
-      <c r="AD1" s="61"/>
-      <c r="AE1" s="61"/>
-      <c r="AF1" s="61"/>
-      <c r="AG1" s="61"/>
-      <c r="AH1" s="59"/>
-      <c r="AI1" s="65" t="s">
+      <c r="AC1" s="63"/>
+      <c r="AD1" s="63"/>
+      <c r="AE1" s="63"/>
+      <c r="AF1" s="63"/>
+      <c r="AG1" s="63"/>
+      <c r="AH1" s="61"/>
+      <c r="AI1" s="68" t="s">
         <v>28</v>
       </c>
-      <c r="AJ1" s="59"/>
-      <c r="AK1" s="58" t="s">
+      <c r="AJ1" s="61"/>
+      <c r="AK1" s="60" t="s">
         <v>29</v>
       </c>
-      <c r="AL1" s="59"/>
-      <c r="AM1" s="60" t="s">
+      <c r="AL1" s="61"/>
+      <c r="AM1" s="62" t="s">
         <v>31</v>
       </c>
-      <c r="AN1" s="61"/>
-      <c r="AO1" s="61"/>
-      <c r="AP1" s="61"/>
-      <c r="AQ1" s="61"/>
-      <c r="AR1" s="59"/>
+      <c r="AN1" s="63"/>
+      <c r="AO1" s="63"/>
+      <c r="AP1" s="63"/>
+      <c r="AQ1" s="63"/>
+      <c r="AR1" s="61"/>
     </row>
     <row r="2" spans="1:44" ht="45.75" customHeight="1">
       <c r="A2" s="16" t="s">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="AO3" s="39">
         <f>(Model!$B$6-AB3)*Model!$B$37</f>
-        <v>9.9999999999999978E-2</v>
+        <v>-9.9999999999999978E-2</v>
       </c>
       <c r="AP3" s="39">
         <f>(AC3-Model!$B$7)*Model!$B$38</f>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="AR3" s="39">
         <f t="shared" ref="AR3:AR11" si="1">SUM(AM3:AQ3)</f>
-        <v>-3.469999999999994</v>
+        <v>-3.6699999999999942</v>
       </c>
     </row>
     <row r="4" spans="1:44" ht="14.25" customHeight="1">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="AO5" s="39">
         <f>(Model!$B$6-AB5)*Model!$B$37</f>
-        <v>-0.20000000000000007</v>
+        <v>0.20000000000000007</v>
       </c>
       <c r="AP5" s="39">
         <f>(AC5-Model!$B$7)*Model!$B$38</f>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="AR5" s="39">
         <f t="shared" si="1"/>
-        <v>-6.7866666666666609</v>
+        <v>-6.3866666666666596</v>
       </c>
     </row>
     <row r="6" spans="1:44" ht="14.25" customHeight="1">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="AO6" s="39">
         <f>(Model!$B$6-AB6)*Model!$B$37</f>
-        <v>0.49999999999999994</v>
+        <v>-0.49999999999999994</v>
       </c>
       <c r="AP6" s="39">
         <f>(AC6-Model!$B$7)*Model!$B$38</f>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="AR6" s="39">
         <f t="shared" si="1"/>
-        <v>-10.029999999999999</v>
+        <v>-11.03</v>
       </c>
     </row>
     <row r="7" spans="1:44" ht="14.25" customHeight="1">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="AO7" s="39">
         <f>(Model!$B$6-AB7)*Model!$B$37</f>
-        <v>0.39999999999999997</v>
+        <v>-0.39999999999999997</v>
       </c>
       <c r="AP7" s="39">
         <f>(AC7-Model!$B$7)*Model!$B$38</f>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="AR7" s="39">
         <f t="shared" si="1"/>
-        <v>-3.7674999999999779</v>
+        <v>-4.5674999999999786</v>
       </c>
     </row>
     <row r="8" spans="1:44" ht="14.25" customHeight="1">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="AO8" s="39">
         <f>(Model!$B$6-AB8)*Model!$B$37</f>
-        <v>0.29999999999999993</v>
+        <v>-0.29999999999999993</v>
       </c>
       <c r="AP8" s="39">
         <f>(AC8-Model!$B$7)*Model!$B$38</f>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="AR8" s="39">
         <f t="shared" si="1"/>
-        <v>-2.6099999999999843</v>
+        <v>-3.209999999999984</v>
       </c>
     </row>
     <row r="9" spans="1:44" ht="14.25" customHeight="1">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="AO9" s="46">
         <f>(Model!$B$6-AB9)*Model!$B$37</f>
-        <v>0.39999999999999997</v>
+        <v>-0.39999999999999997</v>
       </c>
       <c r="AP9" s="46">
         <f>(AC9-Model!$B$7)*Model!$B$38</f>
@@ -2451,7 +2451,7 @@
       </c>
       <c r="AR9" s="46">
         <f t="shared" si="1"/>
-        <v>-1.8149999999999826</v>
+        <v>-2.6149999999999833</v>
       </c>
     </row>
     <row r="10" spans="1:44" ht="14.25" customHeight="1">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="AO10" s="39">
         <f>(Model!$B$6-AB10)*Model!$B$37</f>
-        <v>9.9999999999999978E-2</v>
+        <v>-9.9999999999999978E-2</v>
       </c>
       <c r="AP10" s="39">
         <f>(AC10-Model!$B$7)*Model!$B$38</f>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="AR10" s="39">
         <f t="shared" si="1"/>
-        <v>-3.3333333333333126</v>
+        <v>-3.5333333333333128</v>
       </c>
     </row>
     <row r="11" spans="1:44" ht="14.25" customHeight="1">
@@ -2629,7 +2629,7 @@
         <v>-0.03</v>
       </c>
       <c r="K11" s="28">
-        <v>-0.7</v>
+        <v>-0.6</v>
       </c>
       <c r="L11" s="29">
         <v>2500</v>
@@ -2725,7 +2725,7 @@
       </c>
       <c r="AM11" s="39">
         <f>C11*Model!$B$24+D11*Model!$B$25+E11*Model!$B$26+F11*Model!$B$27+G11*Model!$B$28+H11*Model!$B$29+I11*Model!$B$30+J11*Model!$B$31+K11*Model!$B$32+L11*Model!$B$33</f>
-        <v>5.2</v>
+        <v>1.2</v>
       </c>
       <c r="AN11" s="39">
         <f>(AA11-Model!$B$5)*Model!$B$36</f>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="AO11" s="39">
         <f>(Model!$B$6-AB11)*Model!$B$37</f>
-        <v>-0.7</v>
+        <v>0.7</v>
       </c>
       <c r="AP11" s="39">
         <f>(AC11-Model!$B$7)*Model!$B$38</f>
@@ -2745,7 +2745,7 @@
       </c>
       <c r="AR11" s="39">
         <f t="shared" si="1"/>
-        <v>-12.319999999999958</v>
+        <v>-14.919999999999959</v>
       </c>
     </row>
     <row r="12" spans="1:44" ht="14.25" customHeight="1">
@@ -4227,11 +4227,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="31.5" customHeight="1">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="61"/>
-      <c r="C1" s="59"/>
+      <c r="B1" s="63"/>
+      <c r="C1" s="61"/>
     </row>
     <row r="2" spans="1:3" ht="14.25" customHeight="1">
       <c r="A2" s="1"/>
@@ -4310,11 +4310,11 @@
       <c r="C9" s="8"/>
     </row>
     <row r="10" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A10" s="67" t="s">
+      <c r="A10" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="68"/>
-      <c r="C10" s="69"/>
+      <c r="B10" s="71"/>
+      <c r="C10" s="72"/>
     </row>
     <row r="11" spans="1:3" ht="14.25" customHeight="1">
       <c r="A11" s="8"/>
@@ -4425,11 +4425,11 @@
       <c r="C21" s="8"/>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A22" s="67" t="s">
+      <c r="A22" s="70" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="68"/>
-      <c r="C22" s="69"/>
+      <c r="B22" s="71"/>
+      <c r="C22" s="72"/>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
       <c r="A23" s="9" t="s">
@@ -4532,13 +4532,13 @@
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A32" s="71" t="s">
+      <c r="A32" s="58" t="s">
         <v>102</v>
       </c>
-      <c r="B32" s="72">
-        <v>-10</v>
-      </c>
-      <c r="C32" s="71" t="s">
+      <c r="B32" s="59">
+        <v>-5</v>
+      </c>
+      <c r="C32" s="58" t="s">
         <v>103</v>
       </c>
     </row>
@@ -4559,11 +4559,11 @@
       <c r="C34" s="8"/>
     </row>
     <row r="35" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A35" s="67" t="s">
+      <c r="A35" s="70" t="s">
         <v>59</v>
       </c>
-      <c r="B35" s="68"/>
-      <c r="C35" s="69"/>
+      <c r="B35" s="71"/>
+      <c r="C35" s="72"/>
     </row>
     <row r="36" spans="1:3" ht="14.25" customHeight="1">
       <c r="A36" s="19" t="s">
@@ -4581,7 +4581,7 @@
         <v>63</v>
       </c>
       <c r="B37" s="20">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="C37" s="19" t="s">
         <v>69</v>

</xml_diff>

<commit_message>
fix mc51sd and subs?
</commit_message>
<xml_diff>
--- a/changes/308-ammo-super.xlsx
+++ b/changes/308-ammo-super.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61E7E060-4E14-418B-B6CB-6F2533F36A5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D62D9479-7498-453B-9F23-C524A553A169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="H11" s="27"/>
       <c r="I11" s="25">
-        <v>-900</v>
+        <v>-400</v>
       </c>
       <c r="J11" s="28">
         <v>-0.03</v>
@@ -2711,11 +2711,11 @@
       </c>
       <c r="AI11" s="36">
         <f>Model!$B$4+IF(I11="",0,I11)</f>
-        <v>1170</v>
+        <v>1670</v>
       </c>
       <c r="AJ11" s="32">
         <f t="shared" si="0"/>
-        <v>0.2</v>
+        <v>0.25666666666666665</v>
       </c>
       <c r="AK11" s="37">
         <v>45</v>
@@ -2725,7 +2725,7 @@
       </c>
       <c r="AM11" s="39">
         <f>C11*Model!$B$24+D11*Model!$B$25+E11*Model!$B$26+F11*Model!$B$27+G11*Model!$B$28+H11*Model!$B$29+I11*Model!$B$30+J11*Model!$B$31+K11*Model!$B$32+L11*Model!$B$33</f>
-        <v>1.4000000000000001</v>
+        <v>3.9000000000000004</v>
       </c>
       <c r="AN11" s="39">
         <f>(AA11-Model!$B$5)*Model!$B$36</f>
@@ -2741,11 +2741,11 @@
       </c>
       <c r="AQ11" s="39">
         <f>(AJ11-Model!$B$8)*Model!$B$39</f>
-        <v>-3.2</v>
+        <v>-2.9733333333333336</v>
       </c>
       <c r="AR11" s="39">
         <f t="shared" si="1"/>
-        <v>-14.71999999999996</v>
+        <v>-11.993333333333293</v>
       </c>
     </row>
     <row r="12" spans="1:44" ht="14.25" customHeight="1">

</xml_diff>

<commit_message>
remove 308 subs affecting firerate
</commit_message>
<xml_diff>
--- a/changes/308-ammo-super.xlsx
+++ b/changes/308-ammo-super.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-dev\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D62D9479-7498-453B-9F23-C524A553A169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD54A61-DE80-4262-A99C-78CA285A0B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2625,9 +2625,7 @@
       <c r="I11" s="25">
         <v>-400</v>
       </c>
-      <c r="J11" s="28">
-        <v>-0.03</v>
-      </c>
+      <c r="J11" s="28"/>
       <c r="K11" s="28">
         <v>-0.6</v>
       </c>
@@ -2725,7 +2723,7 @@
       </c>
       <c r="AM11" s="39">
         <f>C11*Model!$B$24+D11*Model!$B$25+E11*Model!$B$26+F11*Model!$B$27+G11*Model!$B$28+H11*Model!$B$29+I11*Model!$B$30+J11*Model!$B$31+K11*Model!$B$32+L11*Model!$B$33</f>
-        <v>3.9000000000000004</v>
+        <v>4.2</v>
       </c>
       <c r="AN11" s="39">
         <f>(AA11-Model!$B$5)*Model!$B$36</f>
@@ -2745,7 +2743,7 @@
       </c>
       <c r="AR11" s="39">
         <f t="shared" si="1"/>
-        <v>-11.993333333333293</v>
+        <v>-11.693333333333293</v>
       </c>
     </row>
     <row r="12" spans="1:44" ht="14.25" customHeight="1">

</xml_diff>